<commit_message>
feat(pipeline): register fresh key 13 in pool, deploy master autonomous sync runner, and ingest week 39 alibra and vv reports
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1990,31 +1990,31 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>NORMAL INTERVAL (Week 39 expected today/tomorrow)</t>
+        <v>1</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="M17" s="2" t="n">
         <v>759</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="O17" s="2" t="n">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
@@ -2028,7 +2028,7 @@
       </c>
       <c r="R17" s="3" t="inlineStr">
         <is>
-          <t>hellenic_alibra_dry_tc_series.csv (6,467 rows)</t>
+          <t>hellenic_alibra_dry_tc_series.csv (6,443 rows)</t>
         </is>
       </c>
       <c r="S17" s="3" t="inlineStr">
@@ -2260,31 +2260,31 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>NORMAL INTERVAL (Week 39 expected today/tomorrow)</t>
+        <v>1</v>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="M20" s="2" t="n">
         <v>757</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>hellenic_alibra_tanker_tc_series.csv (7,191 rows)</t>
+          <t>hellenic_alibra_tanker_tc_series.csv (7,177 rows)</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr">
@@ -2350,31 +2350,31 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>NORMAL INTERVAL</t>
+        <v>2</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
         </is>
       </c>
       <c r="K21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="M21" s="2" t="n">
         <v>726</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="O21" s="2" t="n">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="R21" s="3" t="inlineStr">
         <is>
-          <t>hellenic_vv_matrix_series.csv (12,340 rows), hellenic_vv_sales_series.csv (2,114 rows)</t>
+          <t>hellenic_vv_matrix_series.csv (12,340 rows), hellenic_vv_sales_series.csv (2,122 rows)</t>
         </is>
       </c>
       <c r="S21" s="3" t="inlineStr">
@@ -2710,19 +2710,19 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>NORMAL INTERVAL (Publisher batch releases monthly)</t>
+        <v>7</v>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>CURRENT (Ingested up to Week 39 across DAM 034)</t>
         </is>
       </c>
       <c r="K25" s="2" t="n">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -2731,10 +2731,10 @@
         <v>0</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="O25" s="2" t="n">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
@@ -2743,22 +2743,22 @@
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>Specialized Drewry AIS parser with Executive KPI table (run_drewry_ais.py)</t>
+          <t>Vector PostScript/PDF drawing curve extractor + executive KPI parser (run_drewry_ais_charts.py)</t>
         </is>
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>drewry_ais_fleet_performance_series.csv (14,450 rows), drewry_ais_regional_congestion_series.csv (6,540 rows), drewry_ais_deployment_speed_series.csv (2,448 rows), drewry_ais_utilisation_curves_series.csv (957 rows)</t>
+          <t>drewry_ais_fleet_performance_series.csv (14,768 rows), drewry_ais_regional_congestion_series.csv (6,792 rows), drewry_ais_deployment_speed_series.csv (2,427 rows), drewry_ais_utilisation_curves_series.csv (1,007 rows)</t>
         </is>
       </c>
       <c r="S25" s="3" t="inlineStr">
         <is>
-          <t>run_drewry_ais.py</t>
+          <t>run_drewry_ais_charts.py</t>
         </is>
       </c>
       <c r="T25" s="3" t="inlineStr">
         <is>
-          <t>Overhauled to eliminate OCR noise and page break delimiters. 10 vessel classes tracked.</t>
+          <t>24,994 continuous weekly data points across all 10 vessel classes. Overhauled to eliminate OCR noise.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(pipeline): expand master pipeline runner, detailed drewry ais 10-vessel breakdown, and multi-publisher markdown audit
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,25 +480,25 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
     <col width="39" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="47" customWidth="1" min="4" max="4"/>
     <col width="36" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="45" customWidth="1" min="16" max="16"/>
-    <col width="45" customWidth="1" min="17" max="17"/>
-    <col width="45" customWidth="1" min="18" max="18"/>
+    <col width="48" customWidth="1" min="16" max="16"/>
+    <col width="48" customWidth="1" min="17" max="17"/>
+    <col width="48" customWidth="1" min="18" max="18"/>
     <col width="36" customWidth="1" min="19" max="19"/>
-    <col width="45" customWidth="1" min="20" max="20"/>
+    <col width="48" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2722,7 +2723,7 @@
         </is>
       </c>
       <c r="K25" s="2" t="n">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -2731,10 +2732,10 @@
         <v>0</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="O25" s="2" t="n">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
@@ -2758,7 +2759,7 @@
       </c>
       <c r="T25" s="3" t="inlineStr">
         <is>
-          <t>24,994 continuous weekly data points across all 10 vessel classes. Overhauled to eliminate OCR noise.</t>
+          <t>24,994 continuous weekly data points across all 10 vessel classes: Product LR1 (34), VLCC (32), LPG Carrier (32), Aframax (31), Product LR2 (31), Suezmax (30), Capesize (27), Handysize (25), Panamax (23), Supramax (23).</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2906,7 @@
         <v>10</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>1885</v>
@@ -2928,7 +2929,7 @@
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>signal_reports_metadata.csv (442 rows), data/views/signal/live_fleet_positions.json</t>
+          <t>signal_reports_metadata.csv (446 rows), data/views/signal/live_fleet_positions.json</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr">
@@ -3139,8 +3140,8 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3441,7 +3442,1771 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>signal_reports_metadata.csv (442 rows)</t>
+          <t>signal_reports_metadata.csv (446 rows)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="47" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Domain / Sector</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-Sector / Vessel Class</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Documents / Issues</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Primary Metrics Covered</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Master Series Target CSV</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Total Rows / Points</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Processing Script</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Markdown / Digest Folder</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Capesize (180,000 DWT)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>27 weekly PDFs</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Fleet utilisation %, tonne-miles, ballast speed, Port Hedland/Tubarao delays</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_fleet_performance_series.csv</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>14,768 rows across classes</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/drewry/ais/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Panamax / Kamsarmax (82,000 DWT)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>23 weekly PDFs</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Fleet utilisation %, tonne-miles, ballast speed, Santos/Mississippi delays</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_fleet_performance_series.csv</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>14,768 rows across classes</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/drewry/ais/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Supramax / Ultramax (64,000 DWT)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>23 weekly PDFs</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Fleet utilisation %, tonne-miles, ballast speed, Indonesian coal delays</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_fleet_performance_series.csv</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>14,768 rows across classes</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/drewry/ais/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Handysize (38,000 DWT)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>25 weekly PDFs</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Fleet utilisation %, tonne-miles, ballast speed, minor bulk port queues</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_fleet_performance_series.csv</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>14,768 rows across classes</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/drewry/ais/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>VLCC (300,000 DWT)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>32 weekly PDFs</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Crude utilisation %, tonne-miles, Ras Tanura/Ningbo congestion, ballast speed</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_fleet_performance_series.csv</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>14,768 rows across classes</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/drewry/ais/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Suezmax (160,000 DWT)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>30 weekly PDFs</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Crude utilisation %, tonne-miles, West Africa/Mediterranean queues</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_fleet_performance_series.csv</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>14,768 rows across classes</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/drewry/ais/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Aframax (115,000 DWT)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>31 weekly PDFs</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Dirty utilisation %, tonne-miles, North Sea/Baltic/Caribs queues</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_fleet_performance_series.csv</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>14,768 rows across classes</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/drewry/ais/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Product LR2 (115,000 DWT)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>31 weekly PDFs</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Clean product utilisation %, tonne-miles, MEG-East product flows</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_fleet_performance_series.csv</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>14,768 rows across classes</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/drewry/ais/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Product LR1 (75,000 DWT)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>34 weekly PDFs</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Clean product utilisation %, tonne-miles, regional refinery flows</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_fleet_performance_series.csv</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>14,768 rows across classes</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/drewry/ais/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>LPG Carrier (84,000 CBM VLGC)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>32 weekly PDFs</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>LPG carrier utilisation %, tonne-miles, US Gulf/Ras Laffan flows</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_fleet_performance_series.csv</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>14,768 rows across classes</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/drewry/ais/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Regional Port Congestion (All Classes)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>288 reports</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector curves</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Port waiting days &amp; congestion indexes across China, AG, USG, Aus, Bra</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_regional_congestion_series.csv</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>6,792 rows</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/series/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Deployment &amp; Ballast Speeds (All Classes)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>288 reports</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector curves</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Laden vs ballast cruising speed knots by vessel class and region</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_deployment_speed_series.csv</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2,427 rows</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/series/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Drewry Maritime AIS</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Capacity Utilisation Curves (All Classes)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>288 reports</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>PDF vector curves</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Multi-year historical utilisation curves (2020-2026)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>drewry_ais_utilisation_curves_series.csv</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>1,007 rows</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>run_drewry_ais_charts.py</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/series/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Hellenic Demolition</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Athenian Shipbrokers Cash Buyer</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>1,272 reports</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>HTML / PDF</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Scrap indicative prices ($/LDT) for Bangladesh, India, Pakistan, Turkey</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>hellenic_athenian_demolition_series.csv</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>3,052 rows</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>run_athenian_demolition.py</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/hellenic/demolition/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Hellenic Demolition</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>GMS Weekly Recycler Insights &amp; Deals</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>1,272 reports</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>HTML / PDF</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Cash buyer commentary, scrap sentiment, fixture deals</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>hellenic_gms_demolition_series.csv</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>1,092 rows</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>run_gms_demolition.py</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/hellenic/demolition/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Hellenic Demolition</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>GMS Port Position Queues</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>1,272 reports</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>HTML tables / Images</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Cash buyer port arrivals, beaching positions, tonnage queued</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>hellenic_gms_port_positions_series.csv</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2,905 rows</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>run_gms_demolition.py</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/hellenic/demolition/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Hellenic Demolition</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Best Oasis Scrap Assessments &amp; Deals</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>1,272 reports</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>HTML / PDF</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Subcontinent scrap rates and beaching transaction fixtures</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>hellenic_best_oasis_deals_series.csv</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>882 rows (deals), 859 rows (rates)</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>run_best_oasis_demolition.py</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/hellenic/demolition/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Hellenic Dry Charter</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Alibra Dry Bulk Time Charter Estimates</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>266 reports</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>HTML / Images</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>1Y, 2Y, 3Y, 5Y period TC ($/day) for Capesize, Kamsarmax, Ultramax, Handy</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>hellenic_alibra_dry_tc_series.csv</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>6,443 rows</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>run_hellenic_alibra_tc.py</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/hellenic/dry_charter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Hellenic Tanker Charter</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Alibra Tanker Time Charter Estimates</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>265 reports</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>HTML / Images</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>1Y, 2Y, 3Y, 5Y period TC ($/day) for VLCC, Suezmax, Aframax, LR2, LR1, MR</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>hellenic_alibra_tanker_tc_series.csv</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>7,177 rows</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>run_hellenic_alibra_tc.py</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/hellenic/tanker_charter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Hellenic Iron Ore</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>MMI Daily Brand Price Assessments</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>3,537 reports</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>PDF / HTML</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>31+ brand prices $/dmtu (PB Fines, Newman, Carajas, Lump/Pellet premiums)</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>hellenic_iron_ore_pdf_brands_series.csv</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>31,272 rows</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>run_hellenic_iron_ore_pdf.py</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/hellenic/iron_ore/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Hellenic Iron Ore</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>SMM Daily Spot Iron Ore Benchmark</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>1,171 reports</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>PDF / HTML</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>62% Fe CFR China daily benchmark and port stock statistics</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>hellenic_iron_ore_daily_series.csv</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>1,171 rows</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>run_smm_iron_ore_daily.py</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/hellenic/iron_ore/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Hellenic Iron Ore</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Baltic Capesize C3 / C5 Freight Rates</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>1,164 reports</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>PDF / HTML</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Tubarao-Qingdao (C3) &amp; Dampier-Qingdao (C5) freight $/ton</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>hellenic_capesize_c3_c5_series.csv</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>1,164 rows</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>run_hellenic_iron_ore_pdf.py</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/hellenic/iron_ore/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Hellenic Valuations</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>VesselsValue Secondhand Valuation Matrix</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>261 reports</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>HTML tables / Images</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Resale, 5Y, 10Y, 15Y, 20Y values ($M) for Bulkers, Tankers, Containers</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>hellenic_vv_matrix_series.csv</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>12,340 rows</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>run_hellenic_vv_matrix.py</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/hellenic/vessel_valuations/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Hellenic Valuations</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>VesselsValue Secondhand Sales Deals</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>261 reports</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>HTML tables</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Reported S&amp;P transactions with vessel name, DWT, built, yard, price $M</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>hellenic_vv_sales_series.csv</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>2,122 rows</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>run_hellenic_vessel_valuations.py</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/hellenic/vessel_valuations/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>SSY Simpson Spence Young</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Atlantic Capesize Index (ACI) &amp; Pacific (PCI)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>530 reports</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>PDF tabular</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Atlantic &amp; Pacific Capesize voyage rate indices &amp; iron ore haul routes</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>data/indices/ (display-linked)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Continuous weekly indices</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>run_ssy_complete.py</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/ssy/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Fearnleys Weekly</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>6-Pillar Weekly Market Intelligence</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>526 reports</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>PDF structured</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Crude/Product tankers, Dry Bulk, Gas, Newbuilding, S&amp;P, Macro</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/series/ (normalized rate cards)</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>526 issues cover-to-cover</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>run_fearnleys_normalized.py</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/fearnleys/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Fearnleys Econometric</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>26 Lead-Indicator Econometric Models</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>26 models</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Vector charts / Excel</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Copper vs Supramax, Coal curve vs P5, Iron Ore vs 5TC, S&amp;P vs 1Y TC</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>fearnleys_md_master_econometric_series.xlsx</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>26 workbook sheets</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>export_fearnleys_md_excel.py</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/series/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Poten &amp; Partners</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Tanker Opinions &amp; Top Charterers Series</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>1,087 reports</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>PDF full text</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Narrative essays + 2005-2026 Top Dirty Spot Charterer annual volume rankings</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>poten_top_charterers_series.csv</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>755 rows (charterers), 1,087 rows (metadata)</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>run_poten.py</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/poten/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Seabrokers Seascope</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Offshore Support Vessels, Rigs &amp; Subsea</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>97 reports</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>PDF monthly</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>North Sea OSV dayrates, rig utilization %, subsea &amp; offshore wind</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>seabrokers_osv_monthly_history_series.csv</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>15,430 rows across 9 series</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>run_seabrokers_llamaparse.py</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/seabrokers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Signal Ocean</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Weekly Monitors, Research &amp; Live Fleet</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>515 reports</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>HTML / Telemetry</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Dry &amp; tanker weekly monitors, trade flows, live fleet positions &amp; queues</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>signal_reports_metadata.csv</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>446 rows + live JSON views</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>run_signal.py</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/signal/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Xclusiv Shipbrokers</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Comprehensive Tabular Market Intelligence</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>271 reports</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>PDF tables (9 pages)</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>S&amp;P sales, scrap deals, secondhand matrix, newbuilding orders</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>xclusiv_sales_series.csv</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>17,737 rows across 5 series</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>run_xclusiv_tables.py</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/xclusiv/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Advanced Shipping</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>S&amp;P, Secondhand Matrices, Demo &amp; NB</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>253 reports</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>PDF tables (10 pages)</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>S&amp;P sales, demolition rates &amp; deals, secondhand valuation matrix</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>advanced_shipping_sales_series.csv</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>18,744 rows across 5 series</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>run_advanced_shipping_tables.py</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/advanced_shipping/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Banchero Costa</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>S&amp;P Deals with IMO Numbers &amp; Newbuilding</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>243 reports</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>PDF tables / LlamaParse</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>S&amp;P deals with verified 7-digit IMO numbers, newbuilding orders &amp; prices</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>bancosta_sales_series.csv</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>5,043 rows across 3 series</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>run_banchero_costa_tables.py</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/banchero_costa/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Intermodal</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Secondhand S&amp;P, Newbuilding, Scrap &amp; Baltic</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>256 reports</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>PDF tables / Vector</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Secondhand sales, newbuilding, scrap $/LDT, Page 3 Baltic curves</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>intermodal_baltic_tc_series.csv</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>20,348 rows across series</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>run_intermodal_full.py</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/intermodal/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Drewry WCI</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>World Container Index (WCI) Freight Benchmarks</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>122 weekly rows</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>HTML / Wayback CDX</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>8 major east-west route benchmarks + composite index $/FEU</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>drewry_wci_historical.csv</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>122 weekly rows (display-linked)</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>fetch_drewry_wci.py</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>data/indices/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Pilbara Ports Authority</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Port Hedland &amp; Dampier Iron Ore Export Throughput</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>493 reports</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>PDF tables</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Monthly export tonnage, destination country breakdowns (China, Japan, Korea)</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>australia_ppa_iron_ore.csv</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>424 monthly rows (display-linked)</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>run_ppa.py</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>data/commodities/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(pipeline): wire incremental orchestrator dedup, expand Drewry AIS 10-vessel audit, and deploy universal markdown normalizer
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -3561,7 +3561,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/ais/</t>
+          <t>data/extracted/md/drewry/ais/Drybulk_Capesize/</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/ais/</t>
+          <t>data/extracted/md/drewry/ais/Drybulk_Panamax/</t>
         </is>
       </c>
     </row>
@@ -3655,7 +3655,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/ais/</t>
+          <t>data/extracted/md/drewry/ais/Drybulk_Supramax/</t>
         </is>
       </c>
     </row>
@@ -3702,7 +3702,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/ais/</t>
+          <t>data/extracted/md/drewry/ais/Drybulk_Handysize/</t>
         </is>
       </c>
     </row>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/ais/</t>
+          <t>data/extracted/md/drewry/ais/Crude_VLCC/</t>
         </is>
       </c>
     </row>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/ais/</t>
+          <t>data/extracted/md/drewry/ais/Crude_Suezmax/</t>
         </is>
       </c>
     </row>
@@ -3843,7 +3843,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/ais/</t>
+          <t>data/extracted/md/drewry/ais/Crude_Aframax/</t>
         </is>
       </c>
     </row>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/ais/</t>
+          <t>data/extracted/md/drewry/ais/Product_LR2/</t>
         </is>
       </c>
     </row>
@@ -3937,7 +3937,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/ais/</t>
+          <t>data/extracted/md/drewry/ais/Product_LR1/</t>
         </is>
       </c>
     </row>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/ais/</t>
+          <t>data/extracted/md/drewry/ais/LPG_FR/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(pipeline): integrate seabrokers and smm iron ore into master runner, harden iron ore writer, and refresh cadence audit
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -482,7 +482,7 @@
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="39" customWidth="1" min="3" max="3"/>
-    <col width="47" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
     <col width="36" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
@@ -497,7 +497,7 @@
     <col width="48" customWidth="1" min="16" max="16"/>
     <col width="48" customWidth="1" min="17" max="17"/>
     <col width="48" customWidth="1" min="18" max="18"/>
-    <col width="36" customWidth="1" min="19" max="19"/>
+    <col width="48" customWidth="1" min="19" max="19"/>
     <col width="48" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
@@ -2051,17 +2051,17 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Hellenic: Iron Ore (MMI Daily HTML &amp; PDF)</t>
+          <t>Hellenic: Iron Ore (MMI &amp; SMM Daily)</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>corpus/02-hellenic/iron_ore</t>
+          <t>corpus/02-hellenic/iron_ore/pdfs</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/hellenic/iron_ore</t>
+          <t>data/extracted/md/hellenic/iron_ore_pdf</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -2081,19 +2081,19 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (National Day holiday in China Oct 1-7)</t>
+          <t>CURRENT (Harvested 2026-10-02)</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
-        <v>4518</v>
+        <v>4520</v>
       </c>
       <c r="L18" s="2" t="n">
         <v>1200</v>
@@ -2102,34 +2102,34 @@
         <v>3335</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>3537</v>
+        <v>1188</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>9053</v>
+        <v>9055</v>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
-          <t>Yes (Port inventory curves, Chinese mill profit margin models)</t>
+          <t>Yes (4 SMM driver vector charts + MMi inventory/margin curves)</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>PyMuPDF 2D spatial coordinate parser + HTML index parser</t>
+          <t>PyMuPDF 2D spatial coordinate parser + SMM vector chart clipper</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
         <is>
-          <t>hellenic_iron_ore_pdf_brands_series.csv (31,272 rows), hellenic_iron_ore_daily_series.csv (1,171 rows), hellenic_capesize_c3_c5_series.csv (1,164 rows)</t>
+          <t>hellenic_iron_ore_pdf_brands_series.csv (31,470 rows, 21 CSVs total)</t>
         </is>
       </c>
       <c r="S18" s="3" t="inlineStr">
         <is>
-          <t>run_hellenic_iron_ore_pdf.py</t>
+          <t>run_hellenic_iron_ore_pdf.py &amp; run_smm_iron_ore_daily.py</t>
         </is>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>Covers 31,000+ brand assessment rows across PB fines, Newman, Carajas, lump, and pellet premiums.</t>
+          <t>Full dual-pipeline: 6-page MMi cover-to-cover + 1-page SMM Daily with 4 vector chart clips.</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/hellenic/shipbuilding</t>
+          <t>data/extracted/md/hellenic/shipbuilding/clarksons</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -2209,17 +2209,17 @@
       </c>
       <c r="R19" s="3" t="inlineStr">
         <is>
-          <t>clarksons_sales_series.csv (merged)</t>
+          <t>clarksons_snp_sales_series.csv, clarksons_demolition_sales_series.csv, clarksons_macro_series.csv, clarksons_desk_talk_series.csv</t>
         </is>
       </c>
       <c r="S19" s="3" t="inlineStr">
         <is>
-          <t>run_hellenic_shipbuilding.py</t>
+          <t>run_clarksons_hellas_world_class.py</t>
         </is>
       </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>Clarksons Hellas shipyard contracting and orderbook updates.</t>
+          <t>Clarksons Platou Hellas S&amp;P Bulletins extracted cover-to-cover with reported sales, demolition deals, and desk talk.</t>
         </is>
       </c>
     </row>
@@ -2621,19 +2621,19 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>NORMAL INTERVAL (Published with 3-4 week lag, Sep edition covers Aug)</t>
+        <v>31</v>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>CURRENT (Ingested September 2026 issue today)</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
@@ -2642,10 +2642,10 @@
         <v>0</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P24" s="3" t="inlineStr">
         <is>
@@ -2801,15 +2801,15 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (Assessed Thursdays)</t>
+          <t>CURRENT (Assessed 2026-10-01: $4,434/FEU)</t>
         </is>
       </c>
       <c r="K26" s="2" t="n">
@@ -2839,12 +2839,12 @@
       </c>
       <c r="R26" s="3" t="inlineStr">
         <is>
-          <t>drewry_wci_historical.csv (122 weekly rows, display-linked)</t>
+          <t>drewry_wci_historical.csv (119 weekly rows, display-linked), drewry_opinions_metadata.csv (546 rows), drewry_wci_series.csv (5 rows)</t>
         </is>
       </c>
       <c r="S26" s="3" t="inlineStr">
         <is>
-          <t>fetch_drewry_wci.py</t>
+          <t>run_drewry_opinions.py &amp; fetch_drewry_wci.py</t>
         </is>
       </c>
       <c r="T26" s="3" t="inlineStr">
@@ -2929,12 +2929,12 @@
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>signal_reports_metadata.csv (446 rows), data/views/signal/live_fleet_positions.json</t>
+          <t>signal_reports_metadata.csv (446 rows), data/views/signal/live_fleet_positions.json (9,082 tracked hulls), data/views/signal/port_queues_active.json (1,932 ports)</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr">
         <is>
-          <t>sync_live_fleet_pipeline.py</t>
+          <t>run_signal.py &amp; sync_live_fleet_pipeline.py</t>
         </is>
       </c>
       <c r="T27" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(fearnleys-md): integrate delta sync and asset caching into master pipeline, download latest bespoke reports and update series
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1271,31 +1271,31 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (Harvested 2026-10-02)</t>
         </is>
       </c>
       <c r="K9" s="2" t="n">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>2786</v>
+        <v>2827</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>182</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>3144</v>
+        <v>3189</v>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t>fearnleys_md_master_econometric_series.xlsx (6 sheets, 26 lead models), fearnleys_md_vessel_tightness_series.csv (109 rows), fearnleys_md_macro_correlations_series.csv (78 rows), fearnleys_md_coal_futures_spread_series.csv (46 rows)</t>
+          <t>fearnleys_md_master_econometric_series.xlsx (6 sheets, 26 lead models), fearnleys_md_vessel_tightness_series.csv (112 rows), fearnleys_md_macro_correlations_series.csv (78 rows), fearnleys_md_coal_futures_spread_series.csv (47 rows), fearnleys_md_shipment_volumes_series.csv (40 rows)</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>2,786 high-res vector charts extracted and calibrated. First/last pages discarded per rule.</t>
+          <t>2,827 high-res vector charts extracted and calibrated. First/last pages discarded per rule.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(pipeline): integrate SEC filings incremental ingestion and audit into master autonomous pipeline
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -476,14 +476,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T29"/>
+  <dimension ref="A1:T30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="39" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -3120,6 +3120,96 @@
       <c r="T29" s="3" t="inlineStr">
         <is>
           <t>Directly feeds iron ore throughput charts on index.html. Stored in corpus.duckdb.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>companies_sec_filings</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>SEC EDGAR: Listed Shipping &amp; Dry Bulk Corporates (26 Issuers)</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>corpus/10-companies</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>corpus/10-companies</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Continuous / Statutory Filing Triggers (10-K, 20-F, 10-Q, 6-K, Material 8-K)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2014-01-01</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>CURRENT (1,310 standardized Markdown filings across 26 tickers)</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>1310</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>1310</v>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>No (Complete tabular statutory financials, fleet lists, debt notes)</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>sec2md HTML DOM parser + standardized YAML frontmatter normalizer</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="inlineStr">
+        <is>
+          <t>Direct structured Markdown with standardized YAML frontmatter across 26 corporate subdirectories</t>
+        </is>
+      </c>
+      <c r="S30" s="3" t="inlineStr">
+        <is>
+          <t>fetch_sec_filings.py &amp; audit_sec_corpus.py</t>
+        </is>
+      </c>
+      <c r="T30" s="3" t="inlineStr">
+        <is>
+          <t>100% clean Markdown across 26 tickers (VALE, RIO, BHP, FSUGY, SBLK, GOGL, GNK, SB, DSX, SHIP, CTRM, GLBS, EDRY, FRO, INSW, STNG, DHT, TNK, TRMD, ECO, NAT, TNP, ASC, SFL, NVGS, LPG). Zero conversion artifacts. Standardized YAML frontmatter.</t>
         </is>
       </c>
     </row>
@@ -3457,10 +3547,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
@@ -5210,6 +5300,100 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Corporate SEC Filings (Dry Bulk)</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Major Miners &amp; Dry Bulk Owners (VALE, RIO, BHP, SBLK, GOGL, GNK, SB, DSX, SHIP, CTRM, GLBS, EDRY)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>596 filings</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Markdown / Tables</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Annual Reports (10-K, 20-F), Quarterly Reports (10-Q, 6-K), Material 8-Ks</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>corpus/10-companies/</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>596 statutory filings</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>fetch_sec_filings.py</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>corpus/10-companies/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Corporate SEC Filings (Tankers &amp; Gas)</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Crude, Product &amp; Gas Tankers (FRO, INSW, STNG, DHT, TNK, TRMD, ECO, NAT, TNP, ASC, SFL, NVGS, LPG)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>714 filings</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Markdown / Tables</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Annual Reports (10-K, 20-F), Quarterly Reports (10-Q, 6-K), Material 8-Ks</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>corpus/10-companies/</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>714 statutory filings</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>fetch_sec_filings.py</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>corpus/10-companies/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(pipeline): wire breakwave and baltic automation and enable dynamic cadence audit
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T30"/>
+  <dimension ref="A1:T32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -484,11 +484,11 @@
     <col width="39" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
@@ -549,7 +549,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Status (2026-10-01)</t>
+          <t>Status (2026-10-05)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -641,19 +641,19 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (2d ago)</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>0</v>
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
@@ -679,7 +679,7 @@
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>advanced_shipping_sales_series.csv (6,105 rows), advanced_shipping_demolition_series.csv (2,016 rows), advanced_shipping_secondhand_matrix_series.csv (8,110 rows), advanced_shipping_newbuilding_series.csv (1,909 rows), advanced_shipping_demo_sales_series.csv (604 rows)</t>
+          <t>advanced_shipping_sales_series.csv (6,097 rows), advanced_shipping_demolition_series.csv (2,016 rows), advanced_shipping_secondhand_matrix_series.csv (8,078 rows), advanced_shipping_newbuilding_series.csv (1,895 rows), advanced_shipping_demo_sales_series.csv (601 rows)</t>
         </is>
       </c>
       <c r="S2" s="3" t="inlineStr">
@@ -731,19 +731,19 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="I3" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (2d ago)</t>
         </is>
       </c>
       <c r="K3" s="2" t="n">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>0</v>
@@ -752,10 +752,10 @@
         <v>0</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>affinity_tce_series.csv (4,039 rows), affinity_bda_series.csv (744 rows), affinity_indices_series.csv (490 rows)</t>
+          <t>affinity_tce_series.csv (4,039 rows), affinity_bda_series.csv (744 rows), affinity_indices_series.csv (496 rows)</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr">
@@ -821,19 +821,19 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (Just Ingested W39)</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>0</v>
@@ -842,10 +842,10 @@
         <v>0</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>216</v>
+        <v>433</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
@@ -915,15 +915,15 @@
         </is>
       </c>
       <c r="I5" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (5d ago)</t>
         </is>
       </c>
       <c r="K5" s="2" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>0</v>
@@ -932,10 +932,10 @@
         <v>0</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
@@ -944,22 +944,22 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>Native PyMuPDF table parser (Zero LlamaParse cost for ongoing)</t>
+          <t>LlamaParse cover-to-cover (ciphered/2026) + Native PyMuPDF table &amp; chart parser + clean_all_brokers_formatting.py</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>bancosta_freight_rates_series.csv (20,321 rows), bancosta_ffa_series.csv (7,618 rows), bancosta_sales_series.csv (4,591 rows), bancosta_commodities_series.csv (8,447 rows), bancosta_newbuilding_series.csv (1,952 rows), bancosta_secondhand_matrix_series.csv (1,911 rows), bancosta_demolition_series.csv (1,288 rows)</t>
+          <t>bancosta_freight_rates_series.csv (20,497 rows), bancosta_ffa_series.csv (7,690 rows), bancosta_sales_series.csv (3,220 rows), bancosta_commodities_series.csv (8,519 rows), bancosta_newbuilding_series.csv (2,377 rows), bancosta_secondhand_matrix_series.csv (1,891 rows), bancosta_demolition_series.csv (974 rows)</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>run_banchero_costa_tables.py</t>
+          <t>run_banchero_llamaparse.py &amp; run_banchero_costa_tables.py</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>Extracts exact 7-digit IMO numbers on secondhand vessel transactions. Pages 2 to N-1 parsed.</t>
+          <t>Cover-to-cover LlamaParse for ciphered/2026 reports with automated quality gate (verify_broker_md_quality_gate.py). Extracts exact 7-digit IMO numbers on secondhand vessel transactions. Pages 2 to N-1 parsed.</t>
         </is>
       </c>
     </row>
@@ -1005,11 +1005,11 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
@@ -1022,7 +1022,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>137</v>
+        <v>273</v>
       </c>
       <c r="O6" s="2" t="n">
         <v>136</v>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>carriers_sales_series.csv (3,004 rows), carriers_dry_tc_period_series.csv (3,072 rows), carriers_indices_series.csv (1,792 rows), carriers_tanker_tce_series.csv (768 rows), carriers_bspa_series.csv (713 rows), carriers_newbuilding_series.csv (301 rows), carriers_demolition_series.csv (171 rows)</t>
+          <t>carriers_sales_series.csv (3,130 rows), carriers_dry_tc_period_series.csv (3,216 rows), carriers_indices_series.csv (1,876 rows), carriers_tanker_tce_series.csv (804 rows), carriers_bspa_series.csv (749 rows), carriers_newbuilding_series.csv (312 rows), carriers_demolition_series.csv (178 rows)</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr">
@@ -1091,19 +1091,19 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K7" s="2" t="n">
-        <v>180</v>
+        <v>11</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>0</v>
@@ -1112,10 +1112,10 @@
         <v>0</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>180</v>
+        <v>368</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>180</v>
+        <v>11</v>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
-          <t>clarksons_sales_series.csv (3,920 rows)</t>
+          <t>clarksons_sales_series.csv (1,343 rows)</t>
         </is>
       </c>
       <c r="S7" s="3" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Deduplicated against duplicate uploads on Hellenic portal.</t>
+          <t>Deduplicated against duplicate uploads on Hellenic portal. Week 40 harvested &amp; stacked.</t>
         </is>
       </c>
     </row>
@@ -1181,19 +1181,19 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (Just Ingested W40 Today)</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K8" s="2" t="n">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>0</v>
@@ -1202,10 +1202,10 @@
         <v>0</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>262</v>
+        <v>5005</v>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>fearnleys_rates_series.csv (14,669 rows)</t>
+          <t>fearnleys_rates_series.csv (17,076 rows)</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr">
@@ -1229,44 +1229,44 @@
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>Ingested live today for Week 40 (Sep 30 date). Formatted with 6 distinct pillars.</t>
+          <t>Ingested live for Week 40 (Sep 30 / Oct 02 dates). Formatted with 6 distinct pillars.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>broker_fearnleys_md</t>
+          <t>broker_fearnleys_voice</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Fearnleys-MD (Econometric Research)</t>
+          <t>Fearnleys Broker Voice (Hasura Desk Feeds)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>corpus/01-brokers/fearnleys-md</t>
+          <t>corpus/01-brokers/fearnleys/voice</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/fearnleys-md</t>
+          <t>corpus/01-brokers/fearnleys/voice</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Monthly / Bespoke (Bi-weekly)</t>
+          <t>Weekly (Wednesday-Friday)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Ad-hoc</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>2024-03-25</t>
+          <t>2018-09-05</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1275,285 +1275,285 @@
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (Harvested 2026-10-02)</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K9" s="2" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>2827</v>
+        <v>0</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>182</v>
+        <v>4742</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>3189</v>
+        <v>4742</v>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>Yes (Top 52 econometric recurring lead-indicator models)</t>
+          <t>No (Dense narrative intelligence across 13 desks)</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>Proprietary Dynamic Affine Calibration Engine (R^2 &gt;= 0.999)</t>
+          <t>Direct Hasura GraphQL feed parser with clean Markdown reformatting</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t>fearnleys_md_master_econometric_series.xlsx (6 sheets, 26 lead models), fearnleys_md_vessel_tightness_series.csv (112 rows), fearnleys_md_macro_correlations_series.csv (78 rows), fearnleys_md_coal_futures_spread_series.csv (47 rows), fearnleys_md_shipment_volumes_series.csv (40 rows)</t>
+          <t>fearnleys_broker_comments.csv (11,750 comments), corpus/01-brokers/fearnleys/voice/ (4,744 discrete desk MD files)</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>run_fearnleys_md_full_power.py</t>
+          <t>export_broker_voice_to_corpus.py</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>2,827 high-res vector charts extracted and calibrated. First/last pages discarded per rule.</t>
+          <t>4,744 weekly desk comments segregated by desk and year across 13 desks: Capesize (383), Panamax (383), Supramax (382), VLCC (596), Suezmax (598), Aframax (596), LNG (407), LPG Eastern (342), LPG Western (315), S&amp;P (323), Chartering (392), Gas (24), BLPG (3). Standardized YAML frontmatter.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>broker_intermodal</t>
+          <t>broker_fearnleys_md</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Intermodal Shipbrokers</t>
+          <t>Fearnleys-MD (Econometric Research)</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>corpus/01-brokers/intermodal</t>
+          <t>corpus/01-brokers/fearnleys-md</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/intermodal</t>
+          <t>data/extracted/md/fearnleys-md</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Tuesday)</t>
+          <t>Monthly / Bespoke (Bi-weekly)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Ad-hoc</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2021-06-29</t>
+          <t>2024-03-25</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K10" s="2" t="n">
-        <v>256</v>
+        <v>180</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0</v>
+        <v>2826</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>256</v>
+        <v>183</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>256</v>
+        <v>3191</v>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>Yes (Baltic &amp; Time Charter vector curves, Page 3)</t>
+          <t>Yes (Top 52 econometric recurring lead-indicator models)</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>LlamaParse cover-to-cover + PyMuPDF chart vector curves</t>
+          <t>Proprietary Dynamic Affine Calibration Engine (R^2 &gt;= 0.999)</t>
         </is>
       </c>
       <c r="R10" s="3" t="inlineStr">
         <is>
-          <t>intermodal_baltic_tc_series.csv (20,348 rows), intermodal_tc_rates_series.csv (5,100 rows), intermodal_newbuilding_series.csv (5,058 rows), intermodal_tanker_spot_series.csv (3,879 rows), intermodal_sales_series.csv (3,358 rows), intermodal_demolition_series.csv (2,629 rows)</t>
+          <t>fearnleys_md_master_econometric_series.xlsx (6 sheets, 26 lead models), fearnleys_md_vessel_tightness_series.csv (112 rows), fearnleys_md_macro_correlations_series.csv (78 rows), fearnleys_md_coal_futures_spread_series.csv (47 rows), fearnleys_md_shipment_volumes_series.csv (40 rows)</t>
         </is>
       </c>
       <c r="S10" s="3" t="inlineStr">
         <is>
-          <t>run_intermodal_full.py</t>
+          <t>run_fearnleys_md_full_power.py</t>
         </is>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>100% cover-to-cover extraction (all 8 pages). Editorial essay, Tanker spot, Dry bulk TC, S&amp;P, NB, Demo.</t>
+          <t>2,827 high-res vector charts extracted and calibrated. First/last pages discarded per rule.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>broker_ism</t>
+          <t>broker_gibson</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>ISM Coasters &amp; Mini-Bulkers</t>
+          <t>Gibson Shipbrokers</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>corpus/01-brokers/ism</t>
+          <t>corpus/01-brokers/gibson</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/ism</t>
+          <t>data/extracted/md/gibson</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Monday)</t>
+          <t>Weekly (Friday)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2021-07-05</t>
+          <t>2021-07-02</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="I11" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (10d ago)</t>
         </is>
       </c>
       <c r="K11" s="2" t="n">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="M11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>230</v>
+        <v>264</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>115</v>
+        <v>276</v>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>Yes (4 weekly freight indicator vector charts)</t>
+          <t>Yes (wpDataCharts daily vector curves for all 155 HTML reports in .charts.json)</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>PyMuPDF drawing path &amp; polyline axis scale calibration</t>
+          <t>Native PyMuPDF table parser (PDFs) + BeautifulSoup DOM &amp; wpDataCharts JSON extractor (HTML)</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr">
         <is>
-          <t>ism_handy_freight_series.csv (17,629 rows), ism_coaster_freight_series.csv (12,319 rows)</t>
+          <t>gibson_tanker_spot_series.csv (3,583 rows), gibson_bunker_prices_series.csv (1,011 rows), gibson_master_tanker_series.xlsx</t>
         </is>
       </c>
       <c r="S11" s="3" t="inlineStr">
         <is>
-          <t>run_ism.py</t>
+          <t>run_gibson_pdf.py &amp; run_gibson_html.py</t>
         </is>
       </c>
       <c r="T11" s="3" t="inlineStr">
         <is>
-          <t>Overhauled to eliminate vertical axis tick number chains. Clean commentary under thematic subheaders.</t>
+          <t>100% complete coverage: 109 historical PDFs (2021-2023) + 155 live online HTML reports (2023-2026). Tabular assessments (Spot WS &amp; TCE, FFA, bunkers) and full editorial/sector commentary extracted.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>broker_lion</t>
+          <t>broker_intermodal</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Lion Shipbrokers</t>
+          <t>Intermodal Shipbrokers</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>corpus/01-brokers/lion</t>
+          <t>corpus/01-brokers/intermodal</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/lion</t>
+          <t>data/extracted/md/intermodal</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Friday)</t>
+          <t>Weekly (Tuesday)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2021-07-09</t>
+          <t>2021-06-29</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (5d ago)</t>
         </is>
       </c>
       <c r="K12" s="2" t="n">
-        <v>46</v>
+        <v>257</v>
       </c>
       <c r="L12" s="2" t="n">
         <v>0</v>
@@ -1562,56 +1562,56 @@
         <v>0</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>47</v>
+        <v>258</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>46</v>
+        <v>257</v>
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>No (S&amp;P deals, Demometer indicative ranges, Demo fixtures)</t>
+          <t>Yes (Baltic &amp; Time Charter vector curves, Page 3)</t>
         </is>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>LiteParse in-process layout parser</t>
+          <t>LlamaParse cover-to-cover + PyMuPDF chart vector curves</t>
         </is>
       </c>
       <c r="R12" s="3" t="inlineStr">
         <is>
-          <t>lion_deals_series.csv (1,212 rows), lion_sales_series.csv (1,109 rows), lion_demometer_series.csv (540 rows), lion_demolition_series.csv (516 rows), lion_demo_sales_series.csv (103 rows)</t>
+          <t>intermodal_baltic_tc_series.csv (20,348 rows), intermodal_tc_rates_series.csv (5,233 rows), intermodal_newbuilding_series.csv (5,084 rows), intermodal_tanker_spot_series.csv (3,885 rows), intermodal_sales_series.csv (3,479 rows), intermodal_demolition_series.csv (2,620 rows)</t>
         </is>
       </c>
       <c r="S12" s="3" t="inlineStr">
         <is>
-          <t>run_lion_tables.py</t>
+          <t>run_intermodal_full.py</t>
         </is>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>Joke of the week, author commentary preserved. Disclaimers and contact cards stripped.</t>
+          <t>100% cover-to-cover extraction (all 8 pages). Editorial essay, Tanker spot, Dry bulk TC, S&amp;P, NB, Demo.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>broker_ssy</t>
+          <t>broker_ism</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SSY (Simpson Spence Young)</t>
+          <t>ISM Coasters &amp; Mini-Bulkers</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>corpus/01-brokers/ssy</t>
+          <t>corpus/01-brokers/ism</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/ssy</t>
+          <t>data/extracted/md/ism</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1635,15 +1635,15 @@
         </is>
       </c>
       <c r="I13" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K13" s="2" t="n">
-        <v>530</v>
+        <v>115</v>
       </c>
       <c r="L13" s="2" t="n">
         <v>0</v>
@@ -1652,56 +1652,56 @@
         <v>0</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>531</v>
+        <v>116</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>530</v>
+        <v>115</v>
       </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
-          <t>Yes (Atlantic &amp; Pacific Capesize index vector curves)</t>
+          <t>Yes (4 weekly freight indicator vector charts)</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>PyMuPDF span geometry + vector chart calibration</t>
+          <t>PyMuPDF drawing path &amp; polyline axis scale calibration</t>
         </is>
       </c>
       <c r="R13" s="3" t="inlineStr">
         <is>
-          <t>ssy_capesize_index_series.csv (8,881 rows), ssy_capesize_series.csv (8,881 rows), ssy_route_rates_series.csv (5,190 rows), ssy_capesize_index_time_series.csv (519 rows)</t>
+          <t>ism_handy_freight_series.csv (17,968 rows), ism_coaster_freight_series.csv (12,462 rows)</t>
         </is>
       </c>
       <c r="S13" s="3" t="inlineStr">
         <is>
-          <t>run_ssy_complete.py</t>
+          <t>run_ism.py</t>
         </is>
       </c>
       <c r="T13" s="3" t="inlineStr">
         <is>
-          <t>Covers both Atlantic Capesize Index (ACI) and Pacific Capesize Index (PCI).</t>
+          <t>Overhauled to eliminate vertical axis tick number chains. Clean commentary under thematic subheaders.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>broker_star_asia</t>
+          <t>broker_lion</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Star Asia Demolition</t>
+          <t>Lion Shipbrokers</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>corpus/01-brokers/star_asia</t>
+          <t>corpus/01-brokers/lion</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/star_asia</t>
+          <t>data/extracted/md/lion</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1716,24 +1716,24 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2022-07-22</t>
+          <t>2021-07-09</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K14" s="2" t="n">
-        <v>199</v>
+        <v>48</v>
       </c>
       <c r="L14" s="2" t="n">
         <v>0</v>
@@ -1742,56 +1742,56 @@
         <v>0</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>200</v>
+        <v>96</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>199</v>
+        <v>48</v>
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>Yes (Subcontinent scrap price trends $/LDT, metals/energy)</t>
+          <t>No (S&amp;P deals, Demometer indicative ranges, Demo fixtures)</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>LlamaParse + World-Class Markdown Normalizer (run_star_asia_tables.py)</t>
+          <t>LiteParse in-process layout parser</t>
         </is>
       </c>
       <c r="R14" s="3" t="inlineStr">
         <is>
-          <t>star_asia_snp_sales_series.csv (3,717 rows), star_asia_deals_series.csv (3,327 rows), star_asia_valuation_matrix_series.csv (3,245 rows), star_asia_demolition_series.csv (3,072 rows), star_asia_metals_energy_series.csv (1,327 rows)</t>
+          <t>lion_deals_series.csv (1,269 rows), lion_sales_series.csv (1,164 rows), lion_demometer_series.csv (564 rows), lion_demolition_series.csv (516 rows), lion_demo_sales_series.csv (105 rows)</t>
         </is>
       </c>
       <c r="S14" s="3" t="inlineStr">
         <is>
-          <t>run_star_asia_tables.py</t>
+          <t>run_lion_tables.py</t>
         </is>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>Gaddani / Turkey cell boundary merge defect resolved. Explicit ISO issue dates stamped.</t>
+          <t>Joke of the week, author commentary preserved. Week 40 tables stacked cleanly.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>broker_xclusiv</t>
+          <t>broker_ssy</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Xclusiv Shipbrokers</t>
+          <t>SSY (Simpson Spence Young)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>corpus/01-brokers/xclusiv</t>
+          <t>corpus/01-brokers/ssy</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/xclusiv</t>
+          <t>data/extracted/md/ssy</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>2021-07-26</t>
+          <t>2021-07-05</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1815,15 +1815,15 @@
         </is>
       </c>
       <c r="I15" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K15" s="2" t="n">
-        <v>271</v>
+        <v>530</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
@@ -1832,246 +1832,246 @@
         <v>0</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>271</v>
+        <v>531</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>271</v>
+        <v>530</v>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>Yes (Pages 2-3 freight curves, Pages 8-9 bunker spreads)</t>
+          <t>Yes (Atlantic &amp; Pacific Capesize index vector curves)</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>LiteParse cover-to-cover + vector chart parser</t>
+          <t>PyMuPDF span geometry + vector chart calibration</t>
         </is>
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
-          <t>xclusiv_secondhand_series.csv (8,593 rows), xclusiv_sales_series.csv (5,713 rows), xclusiv_demolition_series.csv (2,098 rows), xclusiv_newbuilding_prices_series.csv (1,397 rows), xclusiv_newbuilding_orders_series.csv (1,329 rows)</t>
+          <t>ssy_capesize_index_series.csv (8,729 rows), ssy_capesize_series.csv (8,881 rows), ssy_route_rates_series.csv (5,160 rows), ssy_capesize_index_time_series.csv (516 rows)</t>
         </is>
       </c>
       <c r="S15" s="3" t="inlineStr">
         <is>
-          <t>run_xclusiv_tables.py</t>
+          <t>run_ssy_complete.py</t>
         </is>
       </c>
       <c r="T15" s="3" t="inlineStr">
         <is>
-          <t>100% cover-to-cover across all 9 pages. Full narrative commentary and S&amp;P tables extracted.</t>
+          <t>Covers both Atlantic Capesize Index (ACI) and Pacific Capesize Index (PCI).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>hellenic_demolition</t>
+          <t>broker_star_asia</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Hellenic: Demolition Market</t>
+          <t>Star Asia Demolition</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>corpus/02-hellenic/demolition</t>
+          <t>corpus/01-brokers/star_asia</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/hellenic/demolition</t>
+          <t>data/extracted/md/star_asia</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Saturday/Sunday)</t>
+          <t>Weekly (Friday)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2014-03-28</t>
+          <t>2022-07-22</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
-        <v>2134</v>
+        <v>199</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>807</v>
+        <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>1208</v>
+        <v>0</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>1272</v>
+        <v>398</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>4149</v>
+        <v>199</v>
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>Yes (Port position queue charts, cash buyer price matrices)</t>
+          <t>Yes (Subcontinent scrap price trends $/LDT, metals/energy)</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>BeautifulSoup HTML + PyMuPDF spatial coordinate table parser</t>
+          <t>LlamaParse + World-Class Markdown Normalizer (run_star_asia_tables.py)</t>
         </is>
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t>hellenic_athenian_demolition_series.csv (3,052 rows), hellenic_gms_port_positions_series.csv (2,905 rows), hellenic_gms_demolition_series.csv (1,092 rows), hellenic_best_oasis_deals_series.csv (882 rows), hellenic_best_oasis_demolition_series.csv (859 rows)</t>
+          <t>star_asia_snp_sales_series.csv (3,575 rows), star_asia_deals_series.csv (3,349 rows), star_asia_valuation_matrix_series.csv (3,232 rows), star_asia_demolition_series.csv (3,120 rows), star_asia_metals_energy_series.csv (1,327 rows)</t>
         </is>
       </c>
       <c r="S16" s="3" t="inlineStr">
         <is>
-          <t>run_hellenic_demolition.py</t>
+          <t>run_star_asia_tables.py</t>
         </is>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>Distinguishes Athenian, Best Oasis, GMS cash buyer reports and port queue tables.</t>
+          <t>Gaddani / Turkey cell boundary merge defect resolved. Explicit ISO issue dates stamped.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>hellenic_dry_charter</t>
+          <t>broker_xclusiv</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Hellenic: Dry Bulk Charter (Alibra)</t>
+          <t>Xclusiv Shipbrokers</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>corpus/02-hellenic/dry_charter</t>
+          <t>corpus/01-brokers/xclusiv</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/hellenic/dry_charter</t>
+          <t>data/extracted/md/xclusiv</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Wednesday)</t>
+          <t>Weekly (Monday)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>2014-03-28</t>
+          <t>2021-07-26</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">
-        <v>0</v>
+        <v>271</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>279</v>
+        <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>759</v>
+        <v>0</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>266</v>
+        <v>536</v>
       </c>
       <c r="O17" s="2" t="n">
-        <v>1038</v>
+        <v>271</v>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>Yes (Alibra rate fixture comparison graphics)</t>
+          <t>Yes (Pages 2-3 freight curves, Pages 8-9 bunker spreads)</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>HTML table &amp; image graphic OCR parsing</t>
+          <t>LiteParse cover-to-cover + vector chart parser</t>
         </is>
       </c>
       <c r="R17" s="3" t="inlineStr">
         <is>
-          <t>hellenic_alibra_dry_tc_series.csv (6,443 rows)</t>
+          <t>xclusiv_secondhand_series.csv (8,529 rows), xclusiv_sales_series.csv (5,542 rows), xclusiv_demolition_series.csv (2,082 rows), xclusiv_newbuilding_prices_series.csv (1,379 rows), xclusiv_newbuilding_orders_series.csv (1,313 rows)</t>
         </is>
       </c>
       <c r="S17" s="3" t="inlineStr">
         <is>
-          <t>run_hellenic_alibra_tc.py</t>
+          <t>run_xclusiv_tables.py</t>
         </is>
       </c>
       <c r="T17" s="3" t="inlineStr">
         <is>
-          <t>Extracts 1Y, 2Y, 3Y, 5Y Dry Bulk period TC assessments across Capesize, Panamax, Supramax, Handy.</t>
+          <t>100% cover-to-cover across all 9 pages. Full narrative commentary and S&amp;P tables extracted.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>hellenic_iron_ore</t>
+          <t>hellenic_demolition</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Hellenic: Iron Ore (MMI &amp; SMM Daily)</t>
+          <t>Hellenic: Demolition Market</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>corpus/02-hellenic/iron_ore/pdfs</t>
+          <t>corpus/02-hellenic/demolition</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/hellenic/iron_ore_pdf</t>
+          <t>data/extracted/md/hellenic/demolition</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Daily (Mon-Fri)</t>
+          <t>Weekly (Saturday/Sunday)</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2081,87 +2081,87 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (Harvested 2026-10-02)</t>
+          <t>CURRENT (2d ago)</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
-        <v>4520</v>
+        <v>2141</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>1200</v>
+        <v>808</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3335</v>
+        <v>1210</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1188</v>
+        <v>1639</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>9055</v>
+        <v>4159</v>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
-          <t>Yes (4 SMM driver vector charts + MMi inventory/margin curves)</t>
+          <t>Yes (Port position queue charts, cash buyer price matrices)</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>PyMuPDF 2D spatial coordinate parser + SMM vector chart clipper</t>
+          <t>BeautifulSoup HTML + PyMuPDF spatial coordinate table parser</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
         <is>
-          <t>hellenic_iron_ore_pdf_brands_series.csv (31,470 rows, 21 CSVs total)</t>
+          <t>hellenic_athenian_demolition_series.csv (2,916 rows), hellenic_gms_port_positions_series.csv (2,921 rows), hellenic_gms_demolition_series.csv (1,096 rows), hellenic_best_oasis_deals_series.csv (892 rows), hellenic_best_oasis_demolition_series.csv (867 rows)</t>
         </is>
       </c>
       <c r="S18" s="3" t="inlineStr">
         <is>
-          <t>run_hellenic_iron_ore_pdf.py &amp; run_smm_iron_ore_daily.py</t>
+          <t>run_hellenic_demolition.py &amp; run_best_oasis_demolition.py &amp; run_gms_demolition.py</t>
         </is>
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>Full dual-pipeline: 6-page MMi cover-to-cover + 1-page SMM Daily with 4 vector chart clips.</t>
+          <t>Distinguishes Athenian, Best Oasis, GMS cash buyer reports and port queue tables. Week 40 stacked.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>hellenic_shipbuilding</t>
+          <t>hellenic_dry_charter</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Hellenic: Shipbuilding &amp; Contracting</t>
+          <t>Hellenic: Dry Bulk Charter (Alibra)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>corpus/02-hellenic/shipbuilding</t>
+          <t>corpus/02-hellenic/dry_charter</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/hellenic/shipbuilding/clarksons</t>
+          <t>data/extracted/md/hellenic/dry_charter</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Friday)</t>
+          <t>Weekly (Wednesday)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -2171,87 +2171,87 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (5d ago)</t>
         </is>
       </c>
       <c r="K19" s="2" t="n">
-        <v>1352</v>
+        <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>379</v>
+        <v>279</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>180</v>
+        <v>760</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>165</v>
+        <v>266</v>
       </c>
       <c r="O19" s="2" t="n">
-        <v>1911</v>
+        <v>1039</v>
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t>No (Shipyard contracting and orderbook tables)</t>
+          <t>Yes (Alibra rate fixture comparison graphics)</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>Native PyMuPDF table parser</t>
+          <t>HTML table &amp; image graphic OCR parsing</t>
         </is>
       </c>
       <c r="R19" s="3" t="inlineStr">
         <is>
-          <t>clarksons_snp_sales_series.csv, clarksons_demolition_sales_series.csv, clarksons_macro_series.csv, clarksons_desk_talk_series.csv</t>
+          <t>hellenic_alibra_dry_tc_series.csv (6,467 rows)</t>
         </is>
       </c>
       <c r="S19" s="3" t="inlineStr">
         <is>
-          <t>run_clarksons_hellas_world_class.py</t>
+          <t>run_hellenic_alibra_tc.py</t>
         </is>
       </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>Clarksons Platou Hellas S&amp;P Bulletins extracted cover-to-cover with reported sales, demolition deals, and desk talk.</t>
+          <t>Extracts 1Y, 2Y, 3Y, 5Y Dry Bulk period TC assessments across Capesize, Panamax, Supramax, Handy.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>hellenic_tanker_charter</t>
+          <t>hellenic_iron_ore</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Hellenic: Tanker Time Charter (Alibra)</t>
+          <t>Hellenic: Iron Ore (MMI &amp; SMM Daily)</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>corpus/02-hellenic/tanker_charter</t>
+          <t>corpus/02-hellenic/iron_ore/pdfs</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/hellenic/tanker_charter</t>
+          <t>data/extracted/md/hellenic/iron_ore_pdf</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Wednesday)</t>
+          <t>Daily (Mon-Fri)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2261,87 +2261,87 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0</v>
+        <v>4523</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>278</v>
+        <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>757</v>
+        <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>265</v>
+        <v>1190</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1035</v>
+        <v>4523</v>
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
-          <t>Yes (Crude &amp; clean period earnings comparison graphics)</t>
+          <t>Yes (4 SMM driver vector charts + MMi inventory/margin curves)</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>HTML table &amp; image graphic OCR parsing</t>
+          <t>PyMuPDF 2D spatial coordinate parser + SMM vector chart clipper</t>
         </is>
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>hellenic_alibra_tanker_tc_series.csv (7,177 rows)</t>
+          <t>hellenic_iron_ore_pdf_brands_series.csv (31,470 rows)</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr">
         <is>
-          <t>run_hellenic_alibra_tc.py</t>
+          <t>run_hellenic_iron_ore_pdf.py &amp; run_smm_iron_ore_daily.py</t>
         </is>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>Extracts 1Y, 2Y, 3Y, 5Y Tanker period TC assessments across VLCC, Suezmax, Aframax, LR2, LR1, MR.</t>
+          <t>Full dual-pipeline: 6-page MMi cover-to-cover + 1-page SMM Daily with 4 vector chart clips.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>hellenic_vessel_valuations</t>
+          <t>hellenic_shipbuilding</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Hellenic: VesselsValue Valuations</t>
+          <t>Hellenic: Shipbuilding &amp; Contracting</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>corpus/02-hellenic/vessel_valuations</t>
+          <t>corpus/02-hellenic/shipbuilding</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/hellenic/vessel_valuations</t>
+          <t>data/extracted/md/hellenic/shipbuilding/clarksons</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Tuesday)</t>
+          <t>Weekly (Friday)</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -2355,363 +2355,363 @@
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K21" s="2" t="n">
-        <v>0</v>
+        <v>1362</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>274</v>
+        <v>379</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>726</v>
+        <v>180</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>261</v>
+        <v>165</v>
       </c>
       <c r="O21" s="2" t="n">
-        <v>1000</v>
+        <v>1921</v>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>Yes (VesselsValue fleet valuation index graphs)</t>
+          <t>No (Shipyard contracting and orderbook tables)</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>HTML table parser + VV valuation matrix calculator</t>
+          <t>Native PyMuPDF table parser</t>
         </is>
       </c>
       <c r="R21" s="3" t="inlineStr">
         <is>
-          <t>hellenic_vv_matrix_series.csv (12,340 rows), hellenic_vv_sales_series.csv (2,122 rows)</t>
+          <t>clarksons_snp_sales_series.csv (1,329 rows), clarksons_demolition_sales_series.csv (70 rows), clarksons_macro_series.csv (165 rows), clarksons_desk_talk_series.csv (352 rows)</t>
         </is>
       </c>
       <c r="S21" s="3" t="inlineStr">
         <is>
-          <t>run_hellenic_vessel_valuations.py</t>
+          <t>run_clarksons_hellas_world_class.py</t>
         </is>
       </c>
       <c r="T21" s="3" t="inlineStr">
         <is>
-          <t>Full secondhand valuation matrix across Bulkers, Tankers, Containers for Newbuilding, 5Y, 10Y, 15Y, 20Y.</t>
+          <t>Clarksons Platou Hellas S&amp;P Bulletins extracted cover-to-cover with reported sales, demolition deals, and desk talk.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>breakwave</t>
+          <t>hellenic_tanker_charter</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Breakwave Advisors</t>
+          <t>Hellenic: Tanker Time Charter (Alibra)</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>corpus/03-breakwave</t>
+          <t>corpus/02-hellenic/tanker_charter</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/breakwave</t>
+          <t>data/extracted/md/hellenic/tanker_charter</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Tuesday) &amp; Daily Insights</t>
+          <t>Weekly (Wednesday)</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2018-07-03</t>
+          <t>2014-03-28</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (5d ago)</t>
         </is>
       </c>
       <c r="K22" s="2" t="n">
-        <v>304</v>
+        <v>0</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>3236</v>
+        <v>278</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>15072</v>
+        <v>758</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>3485</v>
+        <v>265</v>
       </c>
       <c r="O22" s="2" t="n">
-        <v>21806</v>
+        <v>1036</v>
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t>Yes (Dry bulk freight fundamentals &amp; ETF price trajectories)</t>
+          <t>Yes (Crude &amp; clean period earnings comparison graphics)</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>PyMuPDF LiteParse + chart image extraction</t>
+          <t>HTML table &amp; image graphic OCR parsing</t>
         </is>
       </c>
       <c r="R22" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,746 rows), breakwave_insights_metadata.csv (3,194 rows)</t>
+          <t>hellenic_alibra_tanker_tc_series.csv (7,205 rows)</t>
         </is>
       </c>
       <c r="S22" s="3" t="inlineStr">
         <is>
-          <t>run_breakwave_clean_liteparse.py</t>
+          <t>run_hellenic_alibra_tc.py</t>
         </is>
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>15,072 chart images extracted. BDRY and BWET ETF fundamental commentaries parsed.</t>
+          <t>Extracts 1Y, 2Y, 3Y, 5Y Tanker period TC assessments across VLCC, Suezmax, Aframax, LR2, LR1, MR.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>poten</t>
+          <t>hellenic_vessel_valuations</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Poten &amp; Partners (Tanker Opinions)</t>
+          <t>Hellenic: VesselsValue Valuations</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>corpus/04-poten</t>
+          <t>corpus/02-hellenic/vessel_valuations</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/poten</t>
+          <t>data/extracted/md/hellenic/vessel_valuations</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Friday)</t>
+          <t>Weekly (Tuesday)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2004-01-02</t>
+          <t>2014-03-28</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="I23" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>NORMAL INTERVAL (Week 39 due)</t>
+        <v>6</v>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K23" s="2" t="n">
-        <v>1087</v>
+        <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>0</v>
+        <v>274</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0</v>
+        <v>733</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>1087</v>
+        <v>255</v>
       </c>
       <c r="O23" s="2" t="n">
-        <v>3270</v>
+        <v>1007</v>
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>Yes (Top Charterers annual/biannual volume rankings)</t>
+          <t>Yes (VesselsValue fleet valuation index graphs)</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>Local PyMuPDF geometry extraction (poten_clean_v2)</t>
+          <t>HTML table parser + VV valuation matrix calculator</t>
         </is>
       </c>
       <c r="R23" s="3" t="inlineStr">
         <is>
-          <t>poten_opinions_metadata.csv (1,087 rows), poten_top_charterers_series.csv (755 rows), poten_fixtures_series.csv (100 rows)</t>
+          <t>hellenic_vv_matrix_series.csv (12,350 rows), hellenic_vv_sales_series.csv (2,062 rows)</t>
         </is>
       </c>
       <c r="S23" s="3" t="inlineStr">
         <is>
-          <t>run_poten.py</t>
+          <t>run_hellenic_vessel_valuations.py</t>
         </is>
       </c>
       <c r="T23" s="3" t="inlineStr">
         <is>
-          <t>Unbroken 22-year coverage (2004-2026). 1,087 reports cover-to-cover with 0 date exceptions.</t>
+          <t>Full secondhand valuation matrix across Bulkers, Tankers, Containers for Newbuilding, 5Y, 10Y, 15Y, 20Y.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>seabrokers</t>
+          <t>breakwave</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Seabrokers (Seabreeze Monthly Offshore)</t>
+          <t>Breakwave Advisors</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>corpus/05-seabrokers</t>
+          <t>corpus/03-breakwave</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/seabrokers</t>
+          <t>corpus/03-breakwave/insights</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Monthly (1st of Month)</t>
+          <t>Weekly (Tuesday) &amp; Daily Insights</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>1st of Month</t>
+          <t>Tuesday / Daily</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>2018-05-01</t>
+          <t>2018-07-03</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (Ingested September 2026 issue today)</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
-        <v>98</v>
+        <v>304</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>0</v>
+        <v>3239</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>15083</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>98</v>
+        <v>3210</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>196</v>
+        <v>21836</v>
       </c>
       <c r="P24" s="3" t="inlineStr">
         <is>
-          <t>Yes (OSV utilisation curves, rig dayrates, offshore wind)</t>
+          <t>Yes (Dry bulk freight fundamentals, ETF trajectories, &amp; localized Insights charts)</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>LlamaParse cover-to-cover + export_seabrokers_series.py</t>
+          <t>BeautifulSoup DOM + Asset Linker (run_breakwave_insights.py) &amp; PyMuPDF LiteParse (run_breakwave_clean_liteparse.py)</t>
         </is>
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t>seabrokers_osv_monthly_history_series.csv (6,280 rows), seabrokers_rigs_market_series.csv (4,467 rows), seabrokers_osv_utilisation_series.csv (2,304 rows), seabrokers_osv_spot_rates_series.csv (1,855 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,745 rows), breakwave_insights_metadata.csv (3,210 rows)</t>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t>run_seabrokers_llamaparse.py</t>
+          <t>run_breakwave_insights.py &amp; run_breakwave_clean_liteparse.py</t>
         </is>
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>9 master series CSVs (15,430 rows total). Unbroken monthly offshore and subsea coverage.</t>
+          <t>100% 1:1 parity across 3,210 Insights articles (2020-2026) and 291 bi-weekly Dry Bulk/Tanker PDFs. Every article image localized &amp; dual-linked.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>drewry_ais</t>
+          <t>poten</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Drewry Maritime AIS Fleet Performance</t>
+          <t>Poten &amp; Partners (Tanker Opinions)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>corpus/06-drewry/ais</t>
+          <t>corpus/04-poten</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/ais</t>
+          <t>data/extracted/md/poten</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Tuesday)</t>
+          <t>Weekly (Friday)</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2024-01-02</t>
+          <t>2004-01-02</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="I25" s="2" t="n">
@@ -2719,11 +2719,11 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (Ingested up to Week 39 across DAM 034)</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K25" s="2" t="n">
-        <v>288</v>
+        <v>1087</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -2732,88 +2732,88 @@
         <v>0</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>288</v>
+        <v>1087</v>
       </c>
       <c r="O25" s="2" t="n">
-        <v>288</v>
+        <v>1088</v>
       </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
-          <t>Yes (Fleet utilisation, tonne-mile index, bunker fuel price, ballast speeds)</t>
+          <t>Yes (Top Charterers annual/biannual volume rankings)</t>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>Vector PostScript/PDF drawing curve extractor + executive KPI parser (run_drewry_ais_charts.py)</t>
+          <t>Local PyMuPDF geometry extraction (poten_clean_v2)</t>
         </is>
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>drewry_ais_fleet_performance_series.csv (14,768 rows), drewry_ais_regional_congestion_series.csv (6,792 rows), drewry_ais_deployment_speed_series.csv (2,427 rows), drewry_ais_utilisation_curves_series.csv (1,007 rows)</t>
+          <t>poten_opinions_metadata.csv (1,087 rows), poten_top_charterers_series.csv (756 rows), poten_fixtures_series.csv (100 rows)</t>
         </is>
       </c>
       <c r="S25" s="3" t="inlineStr">
         <is>
-          <t>run_drewry_ais_charts.py</t>
+          <t>run_poten.py</t>
         </is>
       </c>
       <c r="T25" s="3" t="inlineStr">
         <is>
-          <t>24,994 continuous weekly data points across all 10 vessel classes: Product LR1 (34), VLCC (32), LPG Carrier (32), Aframax (31), Product LR2 (31), Suezmax (30), Capesize (27), Handysize (25), Panamax (23), Supramax (23).</t>
+          <t>Unbroken 22-year coverage (2004-2026). 1,087 reports cover-to-cover with 0 date exceptions.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>drewry_opinions</t>
+          <t>seabrokers</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Drewry Opinions &amp; World Container Index (WCI)</t>
+          <t>Seabrokers (Seabreeze Monthly Offshore)</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>corpus/06-drewry/opinions</t>
+          <t>corpus/05-seabrokers</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/drewry/opinions</t>
+          <t>data/extracted/md/seabrokers</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Thursday)</t>
+          <t>Monthly (1st of Month)</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>1st of Month</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>2017-11-09</t>
+          <t>2018-05-01</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>CURRENT (Assessed 2026-10-01: $4,434/FEU)</t>
+        <v>34</v>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>NORMAL INTERVAL (34d ago)</t>
         </is>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -2822,71 +2822,71 @@
         <v>0</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>548</v>
+        <v>98</v>
       </c>
       <c r="O26" s="2" t="n">
-        <v>1086</v>
+        <v>197</v>
       </c>
       <c r="P26" s="3" t="inlineStr">
         <is>
-          <t>Yes (Global container freight rate time series)</t>
+          <t>Yes (OSV utilisation curves, rig dayrates, offshore wind)</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>Wayback CDX &amp; live HTML parser with pv18 stability guard</t>
+          <t>LlamaParse cover-to-cover + export_seabrokers_series.py</t>
         </is>
       </c>
       <c r="R26" s="3" t="inlineStr">
         <is>
-          <t>drewry_wci_historical.csv (119 weekly rows, display-linked), drewry_opinions_metadata.csv (546 rows), drewry_wci_series.csv (5 rows)</t>
+          <t>seabrokers_osv_monthly_history_series.csv (6,280 rows), seabrokers_rigs_market_series.csv (5,433 rows), seabrokers_osv_utilisation_series.csv (2,304 rows), seabrokers_osv_spot_rates_series.csv (1,855 rows)</t>
         </is>
       </c>
       <c r="S26" s="3" t="inlineStr">
         <is>
-          <t>run_drewry_opinions.py &amp; fetch_drewry_wci.py</t>
+          <t>run_seabrokers_llamaparse.py</t>
         </is>
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>Contract test verified (38 passed). Displayed directly on index.html.</t>
+          <t>9 master series CSVs (15,430 rows total). Unbroken monthly offshore and subsea coverage.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>signal</t>
+          <t>drewry_ais</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Signal Ocean (Fleet Telemetry &amp; Monitors)</t>
+          <t>Drewry Maritime AIS Fleet Performance</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>corpus/07-signal</t>
+          <t>corpus/06-drewry/ais</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/signal</t>
+          <t>data/extracted/md/drewry/ais</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Friday) &amp; Live Telemetry</t>
+          <t>Weekly (Tuesday)</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>2021-05-14</t>
+          <t>2024-01-02</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2895,319 +2895,499 @@
         </is>
       </c>
       <c r="I27" s="2" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (11d ago)</t>
         </is>
       </c>
       <c r="K27" s="2" t="n">
-        <v>10</v>
+        <v>288</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>515</v>
+        <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>1885</v>
+        <v>0</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>456</v>
+        <v>288</v>
       </c>
       <c r="O27" s="2" t="n">
-        <v>2900</v>
+        <v>289</v>
       </c>
       <c r="P27" s="3" t="inlineStr">
         <is>
-          <t>Yes (Bauxite/Coal/Crude flow monitors, trade flow heatmaps)</t>
+          <t>Yes (Fleet utilisation, tonne-mile index, bunker fuel price, ballast speeds)</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>Playwright session scraper + static monitor markdown builder</t>
+          <t>Vector PostScript/PDF drawing curve extractor + executive KPI parser (run_drewry_ais_charts.py)</t>
         </is>
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>signal_reports_metadata.csv (446 rows), data/views/signal/live_fleet_positions.json (9,082 tracked hulls), data/views/signal/port_queues_active.json (1,932 ports)</t>
+          <t>drewry_ais_fleet_performance_series.csv (14,768 rows), drewry_ais_regional_congestion_series.csv (6,792 rows), drewry_ais_deployment_speed_series.csv (2,427 rows), drewry_ais_utilisation_curves_series.csv (1,007 rows)</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr">
         <is>
-          <t>run_signal.py &amp; sync_live_fleet_pipeline.py</t>
+          <t>run_drewry_ais_charts.py</t>
         </is>
       </c>
       <c r="T27" s="3" t="inlineStr">
         <is>
-          <t>Live automated telemetry syncs active tanker queues and fleet AIS positions.</t>
+          <t>24,994 continuous weekly data points across all 10 vessel classes: Product LR1 (34), VLCC (32), LPG Carrier (32), Aframax (31), Product LR2 (31), Suezmax (30), Capesize (27), Handysize (25), Panamax (23), Supramax (23).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>baltic</t>
+          <t>drewry_opinions</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Baltic Exchange Weekly</t>
+          <t>Drewry Opinions &amp; World Container Index (WCI)</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>corpus/08-baltic</t>
+          <t>corpus/06-drewry/opinions</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>data/extracted/md/baltic</t>
+          <t>data/extracted/md/drewry/opinions</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Weekly (Friday)</t>
+          <t>Weekly (Thursday)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2015-01-02</t>
+          <t>2017-11-09</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="I28" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>3043</v>
+        <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>2218</v>
+        <v>551</v>
       </c>
       <c r="O28" s="2" t="n">
-        <v>5261</v>
+        <v>1097</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
-          <t>No (Detailed fixture narratives and route earnings)</t>
+          <t>Yes (Global container freight rate time series)</t>
         </is>
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>BeautifulSoup HTML layout parser</t>
+          <t>Wayback CDX &amp; live HTML parser with pv18 stability guard</t>
         </is>
       </c>
       <c r="R28" s="3" t="inlineStr">
         <is>
-          <t>baltic_reports_metadata.csv (2,218 rows), baltic_ncfi_series.csv (2,180 rows)</t>
+          <t>drewry_wci_historical.csv (136 rows), drewry_opinions_metadata.csv (551 rows), drewry_wci_series.csv (6 rows)</t>
         </is>
       </c>
       <c r="S28" s="3" t="inlineStr">
         <is>
-          <t>run_baltic.py</t>
+          <t>run_drewry_opinions.py &amp; fetch_drewry_opinions_incremental.py &amp; fetch_drewry_wci.py</t>
         </is>
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>Covers Tanker, Dry Bulk, Container, Gas, and Ningbo Container Freight Index (NCFI).</t>
+          <t>Contract test verified (38 passed). Displayed directly on index.html.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ppa</t>
+          <t>signal</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Pilbara Ports Authority (PPA)</t>
+          <t>Signal Ocean (Fleet Telemetry &amp; Monitors)</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>corpus/09-ppa</t>
+          <t>corpus/07-signal</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>data/commodities</t>
+          <t>data/extracted/md/signal</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Monthly (20th of Month)</t>
+          <t>Weekly (Friday) &amp; Live Telemetry</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>20th of Month</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2016-03-11</t>
+          <t>2021-05-14</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>NORMAL INTERVAL (August throughput figures published late Sep/early Oct)</t>
+        <v>11</v>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>CURRENT (11d ago)</t>
         </is>
       </c>
       <c r="K29" s="2" t="n">
-        <v>493</v>
+        <v>10</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>0</v>
+        <v>515</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0</v>
+        <v>1494</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0</v>
+        <v>446</v>
       </c>
       <c r="O29" s="2" t="n">
-        <v>493</v>
+        <v>2896</v>
       </c>
       <c r="P29" s="3" t="inlineStr">
         <is>
-          <t>No (Port Hedland &amp; Dampier iron ore export tonnage tables)</t>
+          <t>Yes (Bauxite/Coal/Crude flow monitors, trade flow heatmaps)</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>PDF tabular throughput parser + DuckDB</t>
+          <t>Playwright session scraper + static monitor markdown builder</t>
         </is>
       </c>
       <c r="R29" s="3" t="inlineStr">
         <is>
-          <t>australia_ppa_iron_ore.csv (424 rows, display-linked)</t>
+          <t>signal_reports_metadata.csv (446 rows), data/views/signal/live_fleet_positions.json (9,082 tracked hulls), data/views/signal/port_queues_active.json (1,932 ports)</t>
         </is>
       </c>
       <c r="S29" s="3" t="inlineStr">
         <is>
-          <t>run_ppa.py</t>
+          <t>run_signal.py &amp; sync_live_fleet_pipeline.py</t>
         </is>
       </c>
       <c r="T29" s="3" t="inlineStr">
         <is>
-          <t>Directly feeds iron ore throughput charts on index.html. Stored in corpus.duckdb.</t>
+          <t>Live automated telemetry syncs active tanker queues and fleet AIS positions.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>baltic</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Baltic Exchange Weekly</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>corpus/08-baltic</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>corpus/08-baltic</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Weekly (Friday)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2015-01-02</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>CURRENT (3d ago)</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>3047</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>2227</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>5274</v>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>No (Detailed fixture narratives and route earnings)</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>BeautifulSoup HTML layout parser</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="inlineStr">
+        <is>
+          <t>baltic_reports_metadata.csv (2,227 rows), baltic_ncfi_series.csv (2,036 rows)</t>
+        </is>
+      </c>
+      <c r="S30" s="3" t="inlineStr">
+        <is>
+          <t>run_baltic.py</t>
+        </is>
+      </c>
+      <c r="T30" s="3" t="inlineStr">
+        <is>
+          <t>Covers Tanker, Dry Bulk, Container, Gas, and Ningbo Container Freight Index (NCFI). Week 40 (2026-10-02) extracted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>ppa</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Pilbara Ports Authority (PPA)</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>corpus/09-ppa</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>data/commodities</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Monthly (20th of Month)</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>20th of Month</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2016-03-11</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>NORMAL INTERVAL (34d ago)</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>603</v>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>603</v>
+      </c>
+      <c r="P31" s="3" t="inlineStr">
+        <is>
+          <t>No (Port Hedland &amp; Dampier iron ore export tonnage tables)</t>
+        </is>
+      </c>
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>PDF tabular throughput parser + DuckDB</t>
+        </is>
+      </c>
+      <c r="R31" s="3" t="inlineStr">
+        <is>
+          <t>australia_ppa_iron_ore.csv (423 rows)</t>
+        </is>
+      </c>
+      <c r="S31" s="3" t="inlineStr">
+        <is>
+          <t>run_ppa.py</t>
+        </is>
+      </c>
+      <c r="T31" s="3" t="inlineStr">
+        <is>
+          <t>Directly feeds iron ore throughput charts on index.html. Stored in corpus.duckdb.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t>companies_sec_filings</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>SEC EDGAR: Listed Shipping &amp; Dry Bulk Corporates (26 Issuers)</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>corpus/10-companies</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>corpus/10-companies</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>Continuous / Statutory Filing Triggers (10-K, 20-F, 10-Q, 6-K, Material 8-K)</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Continuous</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>2014-01-01</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>CURRENT (1,310 standardized Markdown filings across 26 tickers)</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="2" t="n">
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>CURRENT (3d ago)</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="2" t="n">
         <v>1310</v>
       </c>
-      <c r="O30" s="2" t="n">
+      <c r="O32" s="2" t="n">
         <v>1310</v>
       </c>
-      <c r="P30" s="3" t="inlineStr">
+      <c r="P32" s="3" t="inlineStr">
         <is>
           <t>No (Complete tabular statutory financials, fleet lists, debt notes)</t>
         </is>
       </c>
-      <c r="Q30" s="3" t="inlineStr">
+      <c r="Q32" s="3" t="inlineStr">
         <is>
           <t>sec2md HTML DOM parser + standardized YAML frontmatter normalizer</t>
         </is>
       </c>
-      <c r="R30" s="3" t="inlineStr">
+      <c r="R32" s="3" t="inlineStr">
         <is>
           <t>Direct structured Markdown with standardized YAML frontmatter across 26 corporate subdirectories</t>
         </is>
       </c>
-      <c r="S30" s="3" t="inlineStr">
+      <c r="S32" s="3" t="inlineStr">
         <is>
           <t>fetch_sec_filings.py &amp; audit_sec_corpus.py</t>
         </is>
       </c>
-      <c r="T30" s="3" t="inlineStr">
+      <c r="T32" s="3" t="inlineStr">
         <is>
           <t>100% clean Markdown across 26 tickers (VALE, RIO, BHP, FSUGY, SBLK, GOGL, GNK, SB, DSX, SHIP, CTRM, GLBS, EDRY, FRO, INSW, STNG, DHT, TNK, TRMD, ECO, NAT, TNP, ASC, SFL, NVGS, LPG). Zero conversion artifacts. Standardized YAML frontmatter.</t>
         </is>
@@ -3556,7 +3736,7 @@
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="47" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="48" customWidth="1" min="9" max="9"/>
   </cols>
@@ -3641,7 +3821,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows across classes</t>
+          <t>14,768 rows</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -3688,7 +3868,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows across classes</t>
+          <t>14,768 rows</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -3735,7 +3915,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows across classes</t>
+          <t>14,768 rows</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -3782,7 +3962,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows across classes</t>
+          <t>14,768 rows</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -3829,7 +4009,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows across classes</t>
+          <t>14,768 rows</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3876,7 +4056,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows across classes</t>
+          <t>14,768 rows</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -3923,7 +4103,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows across classes</t>
+          <t>14,768 rows</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -3970,7 +4150,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows across classes</t>
+          <t>14,768 rows</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -4017,7 +4197,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows across classes</t>
+          <t>14,768 rows</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -4064,7 +4244,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows across classes</t>
+          <t>14,768 rows</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -4252,7 +4432,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>3,052 rows</t>
+          <t>2,916 rows</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -4299,7 +4479,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1,092 rows</t>
+          <t>1,096 rows</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -4346,7 +4526,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>2,905 rows</t>
+          <t>2,921 rows</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -4393,7 +4573,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>882 rows (deals), 859 rows (rates)</t>
+          <t>892 rows</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -4440,7 +4620,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>6,443 rows</t>
+          <t>6,467 rows</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -4487,7 +4667,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>7,177 rows</t>
+          <t>7,205 rows</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -4534,7 +4714,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>31,272 rows</t>
+          <t>31,470 rows</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -4581,7 +4761,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>1,171 rows</t>
+          <t>4,770 rows</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -4675,7 +4855,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>12,340 rows</t>
+          <t>12,350 rows</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -4722,7 +4902,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2,122 rows</t>
+          <t>2,062 rows</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -4863,7 +5043,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>26 workbook sheets</t>
+          <t>105 rows</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -4910,7 +5090,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>755 rows (charterers), 1,087 rows (metadata)</t>
+          <t>756 rows</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -4957,7 +5137,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>15,430 rows across 9 series</t>
+          <t>6,280 rows</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -5004,7 +5184,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>446 rows + live JSON views</t>
+          <t>446 rows</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -5051,7 +5231,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>17,737 rows across 5 series</t>
+          <t>5,542 rows</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -5098,7 +5278,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>18,744 rows across 5 series</t>
+          <t>6,097 rows</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -5145,7 +5325,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>5,043 rows across 3 series</t>
+          <t>3,220 rows</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -5192,7 +5372,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>20,348 rows across series</t>
+          <t>20,348 rows</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -5239,7 +5419,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>122 weekly rows (display-linked)</t>
+          <t>136 rows</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -5286,7 +5466,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>424 monthly rows (display-linked)</t>
+          <t>423 rows</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">

</xml_diff>

<commit_message>
fix(md-partition-and-fearnleys-voice): organize extracted md into year subdirs and export fearnleys comments across all sectors
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -842,7 +842,7 @@
         <v>0</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>433</v>
+        <v>219</v>
       </c>
       <c r="O4" s="2" t="n">
         <v>219</v>
@@ -932,7 +932,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="O5" s="2" t="n">
         <v>248</v>
@@ -949,7 +949,7 @@
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>bancosta_freight_rates_series.csv (20,497 rows), bancosta_ffa_series.csv (7,690 rows), bancosta_sales_series.csv (3,220 rows), bancosta_commodities_series.csv (8,519 rows), bancosta_newbuilding_series.csv (2,377 rows), bancosta_secondhand_matrix_series.csv (1,891 rows), bancosta_demolition_series.csv (974 rows)</t>
+          <t>bancosta_freight_rates_series.csv (20,587 rows), bancosta_ffa_series.csv (7,726 rows), bancosta_sales_series.csv (3,220 rows), bancosta_commodities_series.csv (8,555 rows), bancosta_newbuilding_series.csv (2,377 rows), bancosta_secondhand_matrix_series.csv (1,898 rows), bancosta_demolition_series.csv (974 rows)</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
@@ -1022,7 +1022,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>273</v>
+        <v>137</v>
       </c>
       <c r="O6" s="2" t="n">
         <v>136</v>
@@ -1112,7 +1112,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>368</v>
+        <v>188</v>
       </c>
       <c r="O7" s="2" t="n">
         <v>11</v>
@@ -1202,10 +1202,10 @@
         <v>0</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>522</v>
+        <v>12000</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>5005</v>
+        <v>16744</v>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>corpus/01-brokers/fearnleys/voice</t>
+          <t>data/extracted/md/fearnleys/voice</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1292,14 +1292,14 @@
         <v>0</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>4742</v>
+        <v>11739</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>4742</v>
+        <v>16481</v>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>No (Dense narrative intelligence across 13 desks)</t>
+          <t>No (Dense narrative intelligence across 35 desks &amp; routes)</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t>fearnleys_broker_comments.csv (11,750 comments), corpus/01-brokers/fearnleys/voice/ (4,744 discrete desk MD files)</t>
+          <t>fearnleys_broker_comments.csv (11,750 comments), corpus/01-brokers/fearnleys/voice/ (11,750 files), data/extracted/md/fearnleys/voice/ (11,750 files)</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>4,744 weekly desk comments segregated by desk and year across 13 desks: Capesize (383), Panamax (383), Supramax (382), VLCC (596), Suezmax (598), Aframax (596), LNG (407), LPG Eastern (342), LPG Western (315), S&amp;P (323), Chartering (392), Gas (24), BLPG (3). Standardized YAML frontmatter.</t>
+          <t>11,750 weekly desk and route comments segregated by sector, desk, and year across Tankers (8,787), Dry Bulk (1,150), Gas (1,096), Chartering (392), and S&amp;P (325). Standardized YAML frontmatter.</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
         <v>0</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O12" s="2" t="n">
         <v>257</v>
@@ -1652,7 +1652,7 @@
         <v>0</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O13" s="2" t="n">
         <v>115</v>
@@ -1742,7 +1742,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="O14" s="2" t="n">
         <v>48</v>
@@ -1832,7 +1832,7 @@
         <v>0</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="O15" s="2" t="n">
         <v>530</v>
@@ -1922,7 +1922,7 @@
         <v>0</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>398</v>
+        <v>199</v>
       </c>
       <c r="O16" s="2" t="n">
         <v>199</v>
@@ -2012,7 +2012,7 @@
         <v>0</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>536</v>
+        <v>271</v>
       </c>
       <c r="O17" s="2" t="n">
         <v>271</v>

</xml_diff>

<commit_message>
docs(audit): update corpus registry cadence and rag architecture docs
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1139,7 +1139,7 @@
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Deduplicated against duplicate uploads on Hellenic portal. Week 40 harvested &amp; stacked.</t>
+          <t>Clarksons Platou Hellas S&amp;P Bulletins extracted cover-to-cover. Desk Talk commentary properly segregated into distinct dry cargo and tanker sections with Panamax comments preserved. Reported sales, demolition deals, and macro tables stacked.</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
         <v>12000</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>16744</v>
+        <v>5005</v>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>Ingested live for Week 40 (Sep 30 / Oct 02 dates). Formatted with 6 distinct pillars.</t>
+          <t>Ingested live for Week 40. 419 weekly commentary reports generated across all 9 years (2018-2026) in reports/fearnleys/commentary/&lt;year&gt;/ and data/reports/fearnleys/commentary/&lt;year&gt;/. 182 bespoke research reports mirrored into reports/fearnleys/&lt;year&gt;/.</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
         <v>11739</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>16481</v>
+        <v>4742</v>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>Gaddani / Turkey cell boundary merge defect resolved. Explicit ISO issue dates stamped.</t>
+          <t>Gaddani / Turkey cell boundary merge defect resolved. Table headers and Baltic Dry Index / valuation matrices properly labeled. Disclaimers and contact footers removed. Explicit ISO issue dates stamped.</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="T17" s="3" t="inlineStr">
         <is>
-          <t>100% cover-to-cover across all 9 pages. Full narrative commentary and S&amp;P tables extracted.</t>
+          <t>100% cover-to-cover across all 9 pages. Full narrative commentary and S&amp;P tables extracted. Visually audited top pages to guarantee complete commentary and table fidelity without omissions.</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>100% 1:1 parity across 3,210 Insights articles (2020-2026) and 291 bi-weekly Dry Bulk/Tanker PDFs. Every article image localized &amp; dual-linked.</t>
+          <t>100% 1:1 parity across 3,210 Insights articles (2020-2026) and 291 bi-weekly Dry Bulk/Tanker PDFs. Drybulk and Tankers partitioned by year (2018-2026 and 2023-2026). CI freshness comparison logic fixed to unblock automated workflow.</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>Contract test verified (38 passed). Displayed directly on index.html.</t>
+          <t>556 opinion reports spanning 10 years (2017-2026) synchronized into reports/drewry/opinions/&lt;year&gt;/ and corpus/06-drewry/opinions/&lt;year&gt;/. Scraper updated with automatic ISO date prefixing (YYYY-MM-DD_&lt;slug&gt;.md) and dual-saving into both corpus/ and reports/ mirrors. Displayed directly on index.html.</t>
         </is>
       </c>
     </row>
@@ -3263,7 +3263,7 @@
         </is>
       </c>
       <c r="K31" s="2" t="n">
-        <v>603</v>
+        <v>518</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -3275,7 +3275,7 @@
         <v>0</v>
       </c>
       <c r="O31" s="2" t="n">
-        <v>603</v>
+        <v>518</v>
       </c>
       <c r="P31" s="3" t="inlineStr">
         <is>
@@ -3299,7 +3299,7 @@
       </c>
       <c r="T31" s="3" t="inlineStr">
         <is>
-          <t>Directly feeds iron ore throughput charts on index.html. Stored in corpus.duckdb.</t>
+          <t>All 110 loose PDFs consolidated into corpus/09-ppa/_root_pdfs/, leaving 0 unorganized root files. Directly feeds iron ore throughput charts on index.html. Stored in corpus.duckdb.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(rag): define ingestion modalities storage separation and graph rag substrate
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T32"/>
+  <dimension ref="A1:U32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -489,16 +489,17 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="48" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
     <col width="48" customWidth="1" min="17" max="17"/>
     <col width="48" customWidth="1" min="18" max="18"/>
     <col width="48" customWidth="1" min="19" max="19"/>
     <col width="48" customWidth="1" min="20" max="20"/>
+    <col width="48" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -554,50 +555,55 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PDFs</t>
+          <t>PDFs (Corpus)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>HTML (Corpus)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Images</t>
+          <t>Images (Corpus)</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Markdown</t>
+          <t>Native MD (Corpus)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Total Files</t>
+          <t>Extracted MD (data/extracted)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Total Corpus Files</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>Charts Extracted</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Chart Engine</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Master Series CSVs</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Primary Script</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -662,32 +668,35 @@
         <v>0</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>255</v>
+        <v>0</v>
       </c>
       <c r="O2" s="2" t="n">
         <v>255</v>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="n">
+        <v>255</v>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>Yes (Secondhand valuation matrices &amp; demo trends)</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>Native coordinate grid &amp; affine scale parser</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>advanced_shipping_sales_series.csv (6,097 rows), advanced_shipping_demolition_series.csv (2,016 rows), advanced_shipping_secondhand_matrix_series.csv (8,078 rows), advanced_shipping_newbuilding_series.csv (1,895 rows), advanced_shipping_demo_sales_series.csv (601 rows)</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>run_advanced_shipping_tables.py</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>Last 3 pages discarded per parsing rules (currencies/stocks). European comma/dot decimals normalized.</t>
         </is>
@@ -752,32 +761,35 @@
         <v>0</v>
       </c>
       <c r="N3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="n">
         <v>249</v>
       </c>
-      <c r="O3" s="2" t="n">
+      <c r="P3" s="3" t="n">
         <v>256</v>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>Yes (Baltic Dirty &amp; Clean TCE trajectory curves)</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>Native PyMuPDF card layout geometry</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>affinity_tce_series.csv (4,039 rows), affinity_bda_series.csv (744 rows), affinity_indices_series.csv (496 rows)</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>run_affinity_tables.py</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>Handles negative TCE rates (e.g. TC2 -$4,273). Full tanker commentary preserved.</t>
         </is>
@@ -842,32 +854,35 @@
         <v>0</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>219</v>
+        <v>0</v>
       </c>
       <c r="O4" s="2" t="n">
         <v>219</v>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="n">
+        <v>219</v>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>No (Dense indicator tables across 5 pages)</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>Native layout block parser</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr">
         <is>
           <t>agora_indicators_series.csv (10,002 rows)</t>
         </is>
       </c>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>format_agora_properly.py</t>
         </is>
       </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="U4" s="3" t="inlineStr">
         <is>
           <t>Parsed live right now for Week 39 (24 Sep reference). European decimals normalized.</t>
         </is>
@@ -932,32 +947,35 @@
         <v>0</v>
       </c>
       <c r="N5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2" t="n">
         <v>249</v>
       </c>
-      <c r="O5" s="2" t="n">
+      <c r="P5" s="3" t="n">
         <v>248</v>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>Yes (Freight rates, FFA forward curves, ConTex index)</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr">
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>LlamaParse cover-to-cover (ciphered/2026) + Native PyMuPDF table &amp; chart parser + clean_all_brokers_formatting.py</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
+      <c r="S5" s="3" t="inlineStr">
         <is>
           <t>bancosta_freight_rates_series.csv (20,587 rows), bancosta_ffa_series.csv (7,726 rows), bancosta_sales_series.csv (3,220 rows), bancosta_commodities_series.csv (8,555 rows), bancosta_newbuilding_series.csv (2,377 rows), bancosta_secondhand_matrix_series.csv (1,898 rows), bancosta_demolition_series.csv (974 rows)</t>
         </is>
       </c>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>run_banchero_llamaparse.py &amp; run_banchero_costa_tables.py</t>
         </is>
       </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>Cover-to-cover LlamaParse for ciphered/2026 reports with automated quality gate (verify_broker_md_quality_gate.py). Extracts exact 7-digit IMO numbers on secondhand vessel transactions. Pages 2 to N-1 parsed.</t>
         </is>
@@ -1022,32 +1040,35 @@
         <v>0</v>
       </c>
       <c r="N6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2" t="n">
         <v>137</v>
       </c>
-      <c r="O6" s="2" t="n">
+      <c r="P6" s="3" t="n">
         <v>136</v>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>No (Tabular S&amp;P and Baltic BSPA/BDA indices)</t>
         </is>
       </c>
-      <c r="Q6" s="3" t="inlineStr">
+      <c r="R6" s="3" t="inlineStr">
         <is>
           <t>Native word geometry and dynamic anchor parser</t>
         </is>
       </c>
-      <c r="R6" s="3" t="inlineStr">
+      <c r="S6" s="3" t="inlineStr">
         <is>
           <t>carriers_sales_series.csv (3,130 rows), carriers_dry_tc_period_series.csv (3,216 rows), carriers_indices_series.csv (1,876 rows), carriers_tanker_tce_series.csv (804 rows), carriers_bspa_series.csv (749 rows), carriers_newbuilding_series.csv (312 rows), carriers_demolition_series.csv (178 rows)</t>
         </is>
       </c>
-      <c r="S6" s="3" t="inlineStr">
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>run_carriers_complete.py</t>
         </is>
       </c>
-      <c r="T6" s="3" t="inlineStr">
+      <c r="U6" s="3" t="inlineStr">
         <is>
           <t>Greek public equities &amp; daily quote stripped per rules. En bloc sister-ship prices handled.</t>
         </is>
@@ -1112,32 +1133,35 @@
         <v>0</v>
       </c>
       <c r="N7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="n">
         <v>188</v>
       </c>
-      <c r="O7" s="2" t="n">
+      <c r="P7" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="Q7" s="3" t="inlineStr">
         <is>
           <t>No (Bulker &amp; Tanker reported sales transaction tables)</t>
         </is>
       </c>
-      <c r="Q7" s="3" t="inlineStr">
+      <c r="R7" s="3" t="inlineStr">
         <is>
           <t>Native PyMuPDF table coordinate extractor</t>
         </is>
       </c>
-      <c r="R7" s="3" t="inlineStr">
+      <c r="S7" s="3" t="inlineStr">
         <is>
           <t>clarksons_sales_series.csv (1,343 rows)</t>
         </is>
       </c>
-      <c r="S7" s="3" t="inlineStr">
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>run_clarksons.py</t>
         </is>
       </c>
-      <c r="T7" s="3" t="inlineStr">
+      <c r="U7" s="3" t="inlineStr">
         <is>
           <t>Clarksons Platou Hellas S&amp;P Bulletins extracted cover-to-cover. Desk Talk commentary properly segregated into distinct dry cargo and tanker sections with Panamax comments preserved. Reported sales, demolition deals, and macro tables stacked.</t>
         </is>
@@ -1202,32 +1226,35 @@
         <v>0</v>
       </c>
       <c r="N8" s="2" t="n">
+        <v>4742</v>
+      </c>
+      <c r="O8" s="2" t="n">
         <v>12000</v>
       </c>
-      <c r="O8" s="2" t="n">
+      <c r="P8" s="3" t="n">
         <v>5005</v>
       </c>
-      <c r="P8" s="3" t="inlineStr">
+      <c r="Q8" s="3" t="inlineStr">
         <is>
           <t>Yes (Tanker spot WS, Dry bulk BDI &amp; TC, LPG/LNG)</t>
         </is>
       </c>
-      <c r="Q8" s="3" t="inlineStr">
+      <c r="R8" s="3" t="inlineStr">
         <is>
           <t>Specialized 6-pillar normalized parser (run_fearnleys_normalized.py)</t>
         </is>
       </c>
-      <c r="R8" s="3" t="inlineStr">
+      <c r="S8" s="3" t="inlineStr">
         <is>
           <t>fearnleys_rates_series.csv (17,076 rows)</t>
         </is>
       </c>
-      <c r="S8" s="3" t="inlineStr">
+      <c r="T8" s="3" t="inlineStr">
         <is>
           <t>run_fearnleys_normalized.py</t>
         </is>
       </c>
-      <c r="T8" s="3" t="inlineStr">
+      <c r="U8" s="3" t="inlineStr">
         <is>
           <t>Ingested live for Week 40. 419 weekly commentary reports generated across all 9 years (2018-2026) in reports/fearnleys/commentary/&lt;year&gt;/ and data/reports/fearnleys/commentary/&lt;year&gt;/. 182 bespoke research reports mirrored into reports/fearnleys/&lt;year&gt;/.</t>
         </is>
@@ -1292,32 +1319,35 @@
         <v>0</v>
       </c>
       <c r="N9" s="2" t="n">
+        <v>4742</v>
+      </c>
+      <c r="O9" s="2" t="n">
         <v>11739</v>
       </c>
-      <c r="O9" s="2" t="n">
+      <c r="P9" s="3" t="n">
         <v>4742</v>
       </c>
-      <c r="P9" s="3" t="inlineStr">
+      <c r="Q9" s="3" t="inlineStr">
         <is>
           <t>No (Dense narrative intelligence across 35 desks &amp; routes)</t>
         </is>
       </c>
-      <c r="Q9" s="3" t="inlineStr">
+      <c r="R9" s="3" t="inlineStr">
         <is>
           <t>Direct Hasura GraphQL feed parser with clean Markdown reformatting</t>
         </is>
       </c>
-      <c r="R9" s="3" t="inlineStr">
+      <c r="S9" s="3" t="inlineStr">
         <is>
           <t>fearnleys_broker_comments.csv (11,750 comments), corpus/01-brokers/fearnleys/voice/ (11,750 files), data/extracted/md/fearnleys/voice/ (11,750 files)</t>
         </is>
       </c>
-      <c r="S9" s="3" t="inlineStr">
+      <c r="T9" s="3" t="inlineStr">
         <is>
           <t>export_broker_voice_to_corpus.py</t>
         </is>
       </c>
-      <c r="T9" s="3" t="inlineStr">
+      <c r="U9" s="3" t="inlineStr">
         <is>
           <t>11,750 weekly desk and route comments segregated by sector, desk, and year across Tankers (8,787), Dry Bulk (1,150), Gas (1,096), Chartering (392), and S&amp;P (325). Standardized YAML frontmatter.</t>
         </is>
@@ -1382,32 +1412,35 @@
         <v>2826</v>
       </c>
       <c r="N10" s="2" t="n">
+        <v>184</v>
+      </c>
+      <c r="O10" s="2" t="n">
         <v>183</v>
       </c>
-      <c r="O10" s="2" t="n">
+      <c r="P10" s="3" t="n">
         <v>3191</v>
       </c>
-      <c r="P10" s="3" t="inlineStr">
+      <c r="Q10" s="3" t="inlineStr">
         <is>
           <t>Yes (Top 52 econometric recurring lead-indicator models)</t>
         </is>
       </c>
-      <c r="Q10" s="3" t="inlineStr">
+      <c r="R10" s="3" t="inlineStr">
         <is>
           <t>Proprietary Dynamic Affine Calibration Engine (R^2 &gt;= 0.999)</t>
         </is>
       </c>
-      <c r="R10" s="3" t="inlineStr">
+      <c r="S10" s="3" t="inlineStr">
         <is>
           <t>fearnleys_md_master_econometric_series.xlsx (6 sheets, 26 lead models), fearnleys_md_vessel_tightness_series.csv (112 rows), fearnleys_md_macro_correlations_series.csv (78 rows), fearnleys_md_coal_futures_spread_series.csv (47 rows), fearnleys_md_shipment_volumes_series.csv (40 rows)</t>
         </is>
       </c>
-      <c r="S10" s="3" t="inlineStr">
+      <c r="T10" s="3" t="inlineStr">
         <is>
           <t>run_fearnleys_md_full_power.py</t>
         </is>
       </c>
-      <c r="T10" s="3" t="inlineStr">
+      <c r="U10" s="3" t="inlineStr">
         <is>
           <t>2,827 high-res vector charts extracted and calibrated. First/last pages discarded per rule.</t>
         </is>
@@ -1472,32 +1505,35 @@
         <v>0</v>
       </c>
       <c r="N11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2" t="n">
         <v>264</v>
       </c>
-      <c r="O11" s="2" t="n">
+      <c r="P11" s="3" t="n">
         <v>276</v>
       </c>
-      <c r="P11" s="3" t="inlineStr">
+      <c r="Q11" s="3" t="inlineStr">
         <is>
           <t>Yes (wpDataCharts daily vector curves for all 155 HTML reports in .charts.json)</t>
         </is>
       </c>
-      <c r="Q11" s="3" t="inlineStr">
+      <c r="R11" s="3" t="inlineStr">
         <is>
           <t>Native PyMuPDF table parser (PDFs) + BeautifulSoup DOM &amp; wpDataCharts JSON extractor (HTML)</t>
         </is>
       </c>
-      <c r="R11" s="3" t="inlineStr">
+      <c r="S11" s="3" t="inlineStr">
         <is>
           <t>gibson_tanker_spot_series.csv (3,583 rows), gibson_bunker_prices_series.csv (1,011 rows), gibson_master_tanker_series.xlsx</t>
         </is>
       </c>
-      <c r="S11" s="3" t="inlineStr">
+      <c r="T11" s="3" t="inlineStr">
         <is>
           <t>run_gibson_pdf.py &amp; run_gibson_html.py</t>
         </is>
       </c>
-      <c r="T11" s="3" t="inlineStr">
+      <c r="U11" s="3" t="inlineStr">
         <is>
           <t>100% complete coverage: 109 historical PDFs (2021-2023) + 155 live online HTML reports (2023-2026). Tabular assessments (Spot WS &amp; TCE, FFA, bunkers) and full editorial/sector commentary extracted.</t>
         </is>
@@ -1562,32 +1598,35 @@
         <v>0</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>257</v>
+        <v>0</v>
       </c>
       <c r="O12" s="2" t="n">
         <v>257</v>
       </c>
-      <c r="P12" s="3" t="inlineStr">
+      <c r="P12" s="3" t="n">
+        <v>257</v>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
         <is>
           <t>Yes (Baltic &amp; Time Charter vector curves, Page 3)</t>
         </is>
       </c>
-      <c r="Q12" s="3" t="inlineStr">
+      <c r="R12" s="3" t="inlineStr">
         <is>
           <t>LlamaParse cover-to-cover + PyMuPDF chart vector curves</t>
         </is>
       </c>
-      <c r="R12" s="3" t="inlineStr">
+      <c r="S12" s="3" t="inlineStr">
         <is>
           <t>intermodal_baltic_tc_series.csv (20,348 rows), intermodal_tc_rates_series.csv (5,233 rows), intermodal_newbuilding_series.csv (5,084 rows), intermodal_tanker_spot_series.csv (3,885 rows), intermodal_sales_series.csv (3,479 rows), intermodal_demolition_series.csv (2,620 rows)</t>
         </is>
       </c>
-      <c r="S12" s="3" t="inlineStr">
+      <c r="T12" s="3" t="inlineStr">
         <is>
           <t>run_intermodal_full.py</t>
         </is>
       </c>
-      <c r="T12" s="3" t="inlineStr">
+      <c r="U12" s="3" t="inlineStr">
         <is>
           <t>100% cover-to-cover extraction (all 8 pages). Editorial essay, Tanker spot, Dry bulk TC, S&amp;P, NB, Demo.</t>
         </is>
@@ -1652,32 +1691,35 @@
         <v>0</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>115</v>
+        <v>0</v>
       </c>
       <c r="O13" s="2" t="n">
         <v>115</v>
       </c>
-      <c r="P13" s="3" t="inlineStr">
+      <c r="P13" s="3" t="n">
+        <v>115</v>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
         <is>
           <t>Yes (4 weekly freight indicator vector charts)</t>
         </is>
       </c>
-      <c r="Q13" s="3" t="inlineStr">
+      <c r="R13" s="3" t="inlineStr">
         <is>
           <t>PyMuPDF drawing path &amp; polyline axis scale calibration</t>
         </is>
       </c>
-      <c r="R13" s="3" t="inlineStr">
+      <c r="S13" s="3" t="inlineStr">
         <is>
           <t>ism_handy_freight_series.csv (17,968 rows), ism_coaster_freight_series.csv (12,462 rows)</t>
         </is>
       </c>
-      <c r="S13" s="3" t="inlineStr">
+      <c r="T13" s="3" t="inlineStr">
         <is>
           <t>run_ism.py</t>
         </is>
       </c>
-      <c r="T13" s="3" t="inlineStr">
+      <c r="U13" s="3" t="inlineStr">
         <is>
           <t>Overhauled to eliminate vertical axis tick number chains. Clean commentary under thematic subheaders.</t>
         </is>
@@ -1742,32 +1784,35 @@
         <v>0</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="O14" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="P14" s="3" t="inlineStr">
+      <c r="P14" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>No (S&amp;P deals, Demometer indicative ranges, Demo fixtures)</t>
         </is>
       </c>
-      <c r="Q14" s="3" t="inlineStr">
+      <c r="R14" s="3" t="inlineStr">
         <is>
           <t>LiteParse in-process layout parser</t>
         </is>
       </c>
-      <c r="R14" s="3" t="inlineStr">
+      <c r="S14" s="3" t="inlineStr">
         <is>
           <t>lion_deals_series.csv (1,269 rows), lion_sales_series.csv (1,164 rows), lion_demometer_series.csv (564 rows), lion_demolition_series.csv (516 rows), lion_demo_sales_series.csv (105 rows)</t>
         </is>
       </c>
-      <c r="S14" s="3" t="inlineStr">
+      <c r="T14" s="3" t="inlineStr">
         <is>
           <t>run_lion_tables.py</t>
         </is>
       </c>
-      <c r="T14" s="3" t="inlineStr">
+      <c r="U14" s="3" t="inlineStr">
         <is>
           <t>Joke of the week, author commentary preserved. Week 40 tables stacked cleanly.</t>
         </is>
@@ -1832,32 +1877,35 @@
         <v>0</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>530</v>
+        <v>0</v>
       </c>
       <c r="O15" s="2" t="n">
         <v>530</v>
       </c>
-      <c r="P15" s="3" t="inlineStr">
+      <c r="P15" s="3" t="n">
+        <v>530</v>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
         <is>
           <t>Yes (Atlantic &amp; Pacific Capesize index vector curves)</t>
         </is>
       </c>
-      <c r="Q15" s="3" t="inlineStr">
+      <c r="R15" s="3" t="inlineStr">
         <is>
           <t>PyMuPDF span geometry + vector chart calibration</t>
         </is>
       </c>
-      <c r="R15" s="3" t="inlineStr">
+      <c r="S15" s="3" t="inlineStr">
         <is>
           <t>ssy_capesize_index_series.csv (8,729 rows), ssy_capesize_series.csv (8,881 rows), ssy_route_rates_series.csv (5,160 rows), ssy_capesize_index_time_series.csv (516 rows)</t>
         </is>
       </c>
-      <c r="S15" s="3" t="inlineStr">
+      <c r="T15" s="3" t="inlineStr">
         <is>
           <t>run_ssy_complete.py</t>
         </is>
       </c>
-      <c r="T15" s="3" t="inlineStr">
+      <c r="U15" s="3" t="inlineStr">
         <is>
           <t>Covers both Atlantic Capesize Index (ACI) and Pacific Capesize Index (PCI).</t>
         </is>
@@ -1922,32 +1970,35 @@
         <v>0</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>199</v>
+        <v>0</v>
       </c>
       <c r="O16" s="2" t="n">
         <v>199</v>
       </c>
-      <c r="P16" s="3" t="inlineStr">
+      <c r="P16" s="3" t="n">
+        <v>199</v>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
         <is>
           <t>Yes (Subcontinent scrap price trends $/LDT, metals/energy)</t>
         </is>
       </c>
-      <c r="Q16" s="3" t="inlineStr">
+      <c r="R16" s="3" t="inlineStr">
         <is>
           <t>LlamaParse + World-Class Markdown Normalizer (run_star_asia_tables.py)</t>
         </is>
       </c>
-      <c r="R16" s="3" t="inlineStr">
+      <c r="S16" s="3" t="inlineStr">
         <is>
           <t>star_asia_snp_sales_series.csv (3,575 rows), star_asia_deals_series.csv (3,349 rows), star_asia_valuation_matrix_series.csv (3,232 rows), star_asia_demolition_series.csv (3,120 rows), star_asia_metals_energy_series.csv (1,327 rows)</t>
         </is>
       </c>
-      <c r="S16" s="3" t="inlineStr">
+      <c r="T16" s="3" t="inlineStr">
         <is>
           <t>run_star_asia_tables.py</t>
         </is>
       </c>
-      <c r="T16" s="3" t="inlineStr">
+      <c r="U16" s="3" t="inlineStr">
         <is>
           <t>Gaddani / Turkey cell boundary merge defect resolved. Table headers and Baltic Dry Index / valuation matrices properly labeled. Disclaimers and contact footers removed. Explicit ISO issue dates stamped.</t>
         </is>
@@ -2012,32 +2063,35 @@
         <v>0</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>271</v>
+        <v>0</v>
       </c>
       <c r="O17" s="2" t="n">
         <v>271</v>
       </c>
-      <c r="P17" s="3" t="inlineStr">
+      <c r="P17" s="3" t="n">
+        <v>271</v>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
         <is>
           <t>Yes (Pages 2-3 freight curves, Pages 8-9 bunker spreads)</t>
         </is>
       </c>
-      <c r="Q17" s="3" t="inlineStr">
+      <c r="R17" s="3" t="inlineStr">
         <is>
           <t>LiteParse cover-to-cover + vector chart parser</t>
         </is>
       </c>
-      <c r="R17" s="3" t="inlineStr">
+      <c r="S17" s="3" t="inlineStr">
         <is>
           <t>xclusiv_secondhand_series.csv (8,529 rows), xclusiv_sales_series.csv (5,542 rows), xclusiv_demolition_series.csv (2,082 rows), xclusiv_newbuilding_prices_series.csv (1,379 rows), xclusiv_newbuilding_orders_series.csv (1,313 rows)</t>
         </is>
       </c>
-      <c r="S17" s="3" t="inlineStr">
+      <c r="T17" s="3" t="inlineStr">
         <is>
           <t>run_xclusiv_tables.py</t>
         </is>
       </c>
-      <c r="T17" s="3" t="inlineStr">
+      <c r="U17" s="3" t="inlineStr">
         <is>
           <t>100% cover-to-cover across all 9 pages. Full narrative commentary and S&amp;P tables extracted. Visually audited top pages to guarantee complete commentary and table fidelity without omissions.</t>
         </is>
@@ -2102,32 +2156,35 @@
         <v>1210</v>
       </c>
       <c r="N18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="n">
         <v>1639</v>
       </c>
-      <c r="O18" s="2" t="n">
+      <c r="P18" s="3" t="n">
         <v>4159</v>
       </c>
-      <c r="P18" s="3" t="inlineStr">
+      <c r="Q18" s="3" t="inlineStr">
         <is>
           <t>Yes (Port position queue charts, cash buyer price matrices)</t>
         </is>
       </c>
-      <c r="Q18" s="3" t="inlineStr">
+      <c r="R18" s="3" t="inlineStr">
         <is>
           <t>BeautifulSoup HTML + PyMuPDF spatial coordinate table parser</t>
         </is>
       </c>
-      <c r="R18" s="3" t="inlineStr">
+      <c r="S18" s="3" t="inlineStr">
         <is>
           <t>hellenic_athenian_demolition_series.csv (2,916 rows), hellenic_gms_port_positions_series.csv (2,921 rows), hellenic_gms_demolition_series.csv (1,096 rows), hellenic_best_oasis_deals_series.csv (892 rows), hellenic_best_oasis_demolition_series.csv (867 rows)</t>
         </is>
       </c>
-      <c r="S18" s="3" t="inlineStr">
+      <c r="T18" s="3" t="inlineStr">
         <is>
           <t>run_hellenic_demolition.py &amp; run_best_oasis_demolition.py &amp; run_gms_demolition.py</t>
         </is>
       </c>
-      <c r="T18" s="3" t="inlineStr">
+      <c r="U18" s="3" t="inlineStr">
         <is>
           <t>Distinguishes Athenian, Best Oasis, GMS cash buyer reports and port queue tables. Week 40 stacked.</t>
         </is>
@@ -2192,32 +2249,35 @@
         <v>760</v>
       </c>
       <c r="N19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="2" t="n">
         <v>266</v>
       </c>
-      <c r="O19" s="2" t="n">
+      <c r="P19" s="3" t="n">
         <v>1039</v>
       </c>
-      <c r="P19" s="3" t="inlineStr">
+      <c r="Q19" s="3" t="inlineStr">
         <is>
           <t>Yes (Alibra rate fixture comparison graphics)</t>
         </is>
       </c>
-      <c r="Q19" s="3" t="inlineStr">
+      <c r="R19" s="3" t="inlineStr">
         <is>
           <t>HTML table &amp; image graphic OCR parsing</t>
         </is>
       </c>
-      <c r="R19" s="3" t="inlineStr">
+      <c r="S19" s="3" t="inlineStr">
         <is>
           <t>hellenic_alibra_dry_tc_series.csv (6,467 rows)</t>
         </is>
       </c>
-      <c r="S19" s="3" t="inlineStr">
+      <c r="T19" s="3" t="inlineStr">
         <is>
           <t>run_hellenic_alibra_tc.py</t>
         </is>
       </c>
-      <c r="T19" s="3" t="inlineStr">
+      <c r="U19" s="3" t="inlineStr">
         <is>
           <t>Extracts 1Y, 2Y, 3Y, 5Y Dry Bulk period TC assessments across Capesize, Panamax, Supramax, Handy.</t>
         </is>
@@ -2282,32 +2342,35 @@
         <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="2" t="n">
         <v>1190</v>
       </c>
-      <c r="O20" s="2" t="n">
+      <c r="P20" s="3" t="n">
         <v>4523</v>
       </c>
-      <c r="P20" s="3" t="inlineStr">
+      <c r="Q20" s="3" t="inlineStr">
         <is>
           <t>Yes (4 SMM driver vector charts + MMi inventory/margin curves)</t>
         </is>
       </c>
-      <c r="Q20" s="3" t="inlineStr">
+      <c r="R20" s="3" t="inlineStr">
         <is>
           <t>PyMuPDF 2D spatial coordinate parser + SMM vector chart clipper</t>
         </is>
       </c>
-      <c r="R20" s="3" t="inlineStr">
+      <c r="S20" s="3" t="inlineStr">
         <is>
           <t>hellenic_iron_ore_pdf_brands_series.csv (31,470 rows)</t>
         </is>
       </c>
-      <c r="S20" s="3" t="inlineStr">
+      <c r="T20" s="3" t="inlineStr">
         <is>
           <t>run_hellenic_iron_ore_pdf.py &amp; run_smm_iron_ore_daily.py</t>
         </is>
       </c>
-      <c r="T20" s="3" t="inlineStr">
+      <c r="U20" s="3" t="inlineStr">
         <is>
           <t>Full dual-pipeline: 6-page MMi cover-to-cover + 1-page SMM Daily with 4 vector chart clips.</t>
         </is>
@@ -2372,32 +2435,35 @@
         <v>180</v>
       </c>
       <c r="N21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="2" t="n">
         <v>165</v>
       </c>
-      <c r="O21" s="2" t="n">
+      <c r="P21" s="3" t="n">
         <v>1921</v>
       </c>
-      <c r="P21" s="3" t="inlineStr">
+      <c r="Q21" s="3" t="inlineStr">
         <is>
           <t>No (Shipyard contracting and orderbook tables)</t>
         </is>
       </c>
-      <c r="Q21" s="3" t="inlineStr">
+      <c r="R21" s="3" t="inlineStr">
         <is>
           <t>Native PyMuPDF table parser</t>
         </is>
       </c>
-      <c r="R21" s="3" t="inlineStr">
+      <c r="S21" s="3" t="inlineStr">
         <is>
           <t>clarksons_snp_sales_series.csv (1,329 rows), clarksons_demolition_sales_series.csv (70 rows), clarksons_macro_series.csv (165 rows), clarksons_desk_talk_series.csv (352 rows)</t>
         </is>
       </c>
-      <c r="S21" s="3" t="inlineStr">
+      <c r="T21" s="3" t="inlineStr">
         <is>
           <t>run_clarksons_hellas_world_class.py</t>
         </is>
       </c>
-      <c r="T21" s="3" t="inlineStr">
+      <c r="U21" s="3" t="inlineStr">
         <is>
           <t>Clarksons Platou Hellas S&amp;P Bulletins extracted cover-to-cover with reported sales, demolition deals, and desk talk.</t>
         </is>
@@ -2462,32 +2528,35 @@
         <v>758</v>
       </c>
       <c r="N22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="2" t="n">
         <v>265</v>
       </c>
-      <c r="O22" s="2" t="n">
+      <c r="P22" s="3" t="n">
         <v>1036</v>
       </c>
-      <c r="P22" s="3" t="inlineStr">
+      <c r="Q22" s="3" t="inlineStr">
         <is>
           <t>Yes (Crude &amp; clean period earnings comparison graphics)</t>
         </is>
       </c>
-      <c r="Q22" s="3" t="inlineStr">
+      <c r="R22" s="3" t="inlineStr">
         <is>
           <t>HTML table &amp; image graphic OCR parsing</t>
         </is>
       </c>
-      <c r="R22" s="3" t="inlineStr">
+      <c r="S22" s="3" t="inlineStr">
         <is>
           <t>hellenic_alibra_tanker_tc_series.csv (7,205 rows)</t>
         </is>
       </c>
-      <c r="S22" s="3" t="inlineStr">
+      <c r="T22" s="3" t="inlineStr">
         <is>
           <t>run_hellenic_alibra_tc.py</t>
         </is>
       </c>
-      <c r="T22" s="3" t="inlineStr">
+      <c r="U22" s="3" t="inlineStr">
         <is>
           <t>Extracts 1Y, 2Y, 3Y, 5Y Tanker period TC assessments across VLCC, Suezmax, Aframax, LR2, LR1, MR.</t>
         </is>
@@ -2552,32 +2621,35 @@
         <v>733</v>
       </c>
       <c r="N23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="2" t="n">
         <v>255</v>
       </c>
-      <c r="O23" s="2" t="n">
+      <c r="P23" s="3" t="n">
         <v>1007</v>
       </c>
-      <c r="P23" s="3" t="inlineStr">
+      <c r="Q23" s="3" t="inlineStr">
         <is>
           <t>Yes (VesselsValue fleet valuation index graphs)</t>
         </is>
       </c>
-      <c r="Q23" s="3" t="inlineStr">
+      <c r="R23" s="3" t="inlineStr">
         <is>
           <t>HTML table parser + VV valuation matrix calculator</t>
         </is>
       </c>
-      <c r="R23" s="3" t="inlineStr">
+      <c r="S23" s="3" t="inlineStr">
         <is>
           <t>hellenic_vv_matrix_series.csv (12,350 rows), hellenic_vv_sales_series.csv (2,062 rows)</t>
         </is>
       </c>
-      <c r="S23" s="3" t="inlineStr">
+      <c r="T23" s="3" t="inlineStr">
         <is>
           <t>run_hellenic_vessel_valuations.py</t>
         </is>
       </c>
-      <c r="T23" s="3" t="inlineStr">
+      <c r="U23" s="3" t="inlineStr">
         <is>
           <t>Full secondhand valuation matrix across Bulkers, Tankers, Containers for Newbuilding, 5Y, 10Y, 15Y, 20Y.</t>
         </is>
@@ -2645,29 +2717,32 @@
         <v>3210</v>
       </c>
       <c r="O24" s="2" t="n">
+        <v>3210</v>
+      </c>
+      <c r="P24" s="3" t="n">
         <v>21836</v>
       </c>
-      <c r="P24" s="3" t="inlineStr">
+      <c r="Q24" s="3" t="inlineStr">
         <is>
           <t>Yes (Dry bulk freight fundamentals, ETF trajectories, &amp; localized Insights charts)</t>
         </is>
       </c>
-      <c r="Q24" s="3" t="inlineStr">
+      <c r="R24" s="3" t="inlineStr">
         <is>
           <t>BeautifulSoup DOM + Asset Linker (run_breakwave_insights.py) &amp; PyMuPDF LiteParse (run_breakwave_clean_liteparse.py)</t>
         </is>
       </c>
-      <c r="R24" s="3" t="inlineStr">
+      <c r="S24" s="3" t="inlineStr">
         <is>
           <t>breakwave_fundamentals_series.csv (2,745 rows), breakwave_insights_metadata.csv (3,210 rows)</t>
         </is>
       </c>
-      <c r="S24" s="3" t="inlineStr">
+      <c r="T24" s="3" t="inlineStr">
         <is>
           <t>run_breakwave_insights.py &amp; run_breakwave_clean_liteparse.py</t>
         </is>
       </c>
-      <c r="T24" s="3" t="inlineStr">
+      <c r="U24" s="3" t="inlineStr">
         <is>
           <t>100% 1:1 parity across 3,210 Insights articles (2020-2026) and 291 bi-weekly Dry Bulk/Tanker PDFs. Drybulk and Tankers partitioned by year (2018-2026 and 2023-2026). CI freshness comparison logic fixed to unblock automated workflow.</t>
         </is>
@@ -2732,32 +2807,35 @@
         <v>0</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>1087</v>
+        <v>0</v>
       </c>
       <c r="O25" s="2" t="n">
         <v>1087</v>
       </c>
-      <c r="P25" s="3" t="inlineStr">
+      <c r="P25" s="3" t="n">
+        <v>1087</v>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
         <is>
           <t>Yes (Top Charterers annual/biannual volume rankings)</t>
         </is>
       </c>
-      <c r="Q25" s="3" t="inlineStr">
+      <c r="R25" s="3" t="inlineStr">
         <is>
           <t>Local PyMuPDF geometry extraction (poten_clean_v2)</t>
         </is>
       </c>
-      <c r="R25" s="3" t="inlineStr">
+      <c r="S25" s="3" t="inlineStr">
         <is>
           <t>poten_opinions_metadata.csv (1,087 rows), poten_top_charterers_series.csv (756 rows), poten_fixtures_series.csv (100 rows)</t>
         </is>
       </c>
-      <c r="S25" s="3" t="inlineStr">
+      <c r="T25" s="3" t="inlineStr">
         <is>
           <t>run_poten.py</t>
         </is>
       </c>
-      <c r="T25" s="3" t="inlineStr">
+      <c r="U25" s="3" t="inlineStr">
         <is>
           <t>Unbroken 22-year coverage (2004-2026). 1,087 reports cover-to-cover with 0 date exceptions.</t>
         </is>
@@ -2822,32 +2900,35 @@
         <v>0</v>
       </c>
       <c r="N26" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="O26" s="2" t="n">
         <v>98</v>
       </c>
-      <c r="O26" s="2" t="n">
+      <c r="P26" s="3" t="n">
         <v>197</v>
       </c>
-      <c r="P26" s="3" t="inlineStr">
+      <c r="Q26" s="3" t="inlineStr">
         <is>
           <t>Yes (OSV utilisation curves, rig dayrates, offshore wind)</t>
         </is>
       </c>
-      <c r="Q26" s="3" t="inlineStr">
+      <c r="R26" s="3" t="inlineStr">
         <is>
           <t>LlamaParse cover-to-cover + export_seabrokers_series.py</t>
         </is>
       </c>
-      <c r="R26" s="3" t="inlineStr">
+      <c r="S26" s="3" t="inlineStr">
         <is>
           <t>seabrokers_osv_monthly_history_series.csv (6,280 rows), seabrokers_rigs_market_series.csv (5,433 rows), seabrokers_osv_utilisation_series.csv (2,304 rows), seabrokers_osv_spot_rates_series.csv (1,855 rows)</t>
         </is>
       </c>
-      <c r="S26" s="3" t="inlineStr">
+      <c r="T26" s="3" t="inlineStr">
         <is>
           <t>run_seabrokers_llamaparse.py</t>
         </is>
       </c>
-      <c r="T26" s="3" t="inlineStr">
+      <c r="U26" s="3" t="inlineStr">
         <is>
           <t>9 master series CSVs (15,430 rows total). Unbroken monthly offshore and subsea coverage.</t>
         </is>
@@ -2912,32 +2993,35 @@
         <v>0</v>
       </c>
       <c r="N27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="2" t="n">
         <v>288</v>
       </c>
-      <c r="O27" s="2" t="n">
+      <c r="P27" s="3" t="n">
         <v>289</v>
       </c>
-      <c r="P27" s="3" t="inlineStr">
+      <c r="Q27" s="3" t="inlineStr">
         <is>
           <t>Yes (Fleet utilisation, tonne-mile index, bunker fuel price, ballast speeds)</t>
         </is>
       </c>
-      <c r="Q27" s="3" t="inlineStr">
+      <c r="R27" s="3" t="inlineStr">
         <is>
           <t>Vector PostScript/PDF drawing curve extractor + executive KPI parser (run_drewry_ais_charts.py)</t>
         </is>
       </c>
-      <c r="R27" s="3" t="inlineStr">
+      <c r="S27" s="3" t="inlineStr">
         <is>
           <t>drewry_ais_fleet_performance_series.csv (14,768 rows), drewry_ais_regional_congestion_series.csv (6,792 rows), drewry_ais_deployment_speed_series.csv (2,427 rows), drewry_ais_utilisation_curves_series.csv (1,007 rows)</t>
         </is>
       </c>
-      <c r="S27" s="3" t="inlineStr">
+      <c r="T27" s="3" t="inlineStr">
         <is>
           <t>run_drewry_ais_charts.py</t>
         </is>
       </c>
-      <c r="T27" s="3" t="inlineStr">
+      <c r="U27" s="3" t="inlineStr">
         <is>
           <t>24,994 continuous weekly data points across all 10 vessel classes: Product LR1 (34), VLCC (32), LPG Carrier (32), Aframax (31), Product LR2 (31), Suezmax (30), Capesize (27), Handysize (25), Panamax (23), Supramax (23).</t>
         </is>
@@ -3002,32 +3086,35 @@
         <v>0</v>
       </c>
       <c r="N28" s="2" t="n">
+        <v>1092</v>
+      </c>
+      <c r="O28" s="2" t="n">
         <v>551</v>
       </c>
-      <c r="O28" s="2" t="n">
+      <c r="P28" s="3" t="n">
         <v>1097</v>
       </c>
-      <c r="P28" s="3" t="inlineStr">
+      <c r="Q28" s="3" t="inlineStr">
         <is>
           <t>Yes (Global container freight rate time series)</t>
         </is>
       </c>
-      <c r="Q28" s="3" t="inlineStr">
+      <c r="R28" s="3" t="inlineStr">
         <is>
           <t>Wayback CDX &amp; live HTML parser with pv18 stability guard</t>
         </is>
       </c>
-      <c r="R28" s="3" t="inlineStr">
+      <c r="S28" s="3" t="inlineStr">
         <is>
           <t>drewry_wci_historical.csv (136 rows), drewry_opinions_metadata.csv (551 rows), drewry_wci_series.csv (6 rows)</t>
         </is>
       </c>
-      <c r="S28" s="3" t="inlineStr">
+      <c r="T28" s="3" t="inlineStr">
         <is>
           <t>run_drewry_opinions.py &amp; fetch_drewry_opinions_incremental.py &amp; fetch_drewry_wci.py</t>
         </is>
       </c>
-      <c r="T28" s="3" t="inlineStr">
+      <c r="U28" s="3" t="inlineStr">
         <is>
           <t>556 opinion reports spanning 10 years (2017-2026) synchronized into reports/drewry/opinions/&lt;year&gt;/ and corpus/06-drewry/opinions/&lt;year&gt;/. Scraper updated with automatic ISO date prefixing (YYYY-MM-DD_&lt;slug&gt;.md) and dual-saving into both corpus/ and reports/ mirrors. Displayed directly on index.html.</t>
         </is>
@@ -3092,32 +3179,35 @@
         <v>1494</v>
       </c>
       <c r="N29" s="2" t="n">
+        <v>451</v>
+      </c>
+      <c r="O29" s="2" t="n">
         <v>446</v>
       </c>
-      <c r="O29" s="2" t="n">
+      <c r="P29" s="3" t="n">
         <v>2896</v>
       </c>
-      <c r="P29" s="3" t="inlineStr">
+      <c r="Q29" s="3" t="inlineStr">
         <is>
           <t>Yes (Bauxite/Coal/Crude flow monitors, trade flow heatmaps)</t>
         </is>
       </c>
-      <c r="Q29" s="3" t="inlineStr">
+      <c r="R29" s="3" t="inlineStr">
         <is>
           <t>Playwright session scraper + static monitor markdown builder</t>
         </is>
       </c>
-      <c r="R29" s="3" t="inlineStr">
+      <c r="S29" s="3" t="inlineStr">
         <is>
           <t>signal_reports_metadata.csv (446 rows), data/views/signal/live_fleet_positions.json (9,082 tracked hulls), data/views/signal/port_queues_active.json (1,932 ports)</t>
         </is>
       </c>
-      <c r="S29" s="3" t="inlineStr">
+      <c r="T29" s="3" t="inlineStr">
         <is>
           <t>run_signal.py &amp; sync_live_fleet_pipeline.py</t>
         </is>
       </c>
-      <c r="T29" s="3" t="inlineStr">
+      <c r="U29" s="3" t="inlineStr">
         <is>
           <t>Live automated telemetry syncs active tanker queues and fleet AIS positions.</t>
         </is>
@@ -3185,29 +3275,32 @@
         <v>2227</v>
       </c>
       <c r="O30" s="2" t="n">
+        <v>2227</v>
+      </c>
+      <c r="P30" s="3" t="n">
         <v>5274</v>
       </c>
-      <c r="P30" s="3" t="inlineStr">
+      <c r="Q30" s="3" t="inlineStr">
         <is>
           <t>No (Detailed fixture narratives and route earnings)</t>
         </is>
       </c>
-      <c r="Q30" s="3" t="inlineStr">
+      <c r="R30" s="3" t="inlineStr">
         <is>
           <t>BeautifulSoup HTML layout parser</t>
         </is>
       </c>
-      <c r="R30" s="3" t="inlineStr">
+      <c r="S30" s="3" t="inlineStr">
         <is>
           <t>baltic_reports_metadata.csv (2,227 rows), baltic_ncfi_series.csv (2,036 rows)</t>
         </is>
       </c>
-      <c r="S30" s="3" t="inlineStr">
+      <c r="T30" s="3" t="inlineStr">
         <is>
           <t>run_baltic.py</t>
         </is>
       </c>
-      <c r="T30" s="3" t="inlineStr">
+      <c r="U30" s="3" t="inlineStr">
         <is>
           <t>Covers Tanker, Dry Bulk, Container, Gas, and Ningbo Container Freight Index (NCFI). Week 40 (2026-10-02) extracted.</t>
         </is>
@@ -3275,29 +3368,32 @@
         <v>0</v>
       </c>
       <c r="O31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="3" t="n">
         <v>518</v>
       </c>
-      <c r="P31" s="3" t="inlineStr">
+      <c r="Q31" s="3" t="inlineStr">
         <is>
           <t>No (Port Hedland &amp; Dampier iron ore export tonnage tables)</t>
         </is>
       </c>
-      <c r="Q31" s="3" t="inlineStr">
+      <c r="R31" s="3" t="inlineStr">
         <is>
           <t>PDF tabular throughput parser + DuckDB</t>
         </is>
       </c>
-      <c r="R31" s="3" t="inlineStr">
+      <c r="S31" s="3" t="inlineStr">
         <is>
           <t>australia_ppa_iron_ore.csv (423 rows)</t>
         </is>
       </c>
-      <c r="S31" s="3" t="inlineStr">
+      <c r="T31" s="3" t="inlineStr">
         <is>
           <t>run_ppa.py</t>
         </is>
       </c>
-      <c r="T31" s="3" t="inlineStr">
+      <c r="U31" s="3" t="inlineStr">
         <is>
           <t>All 110 loose PDFs consolidated into corpus/09-ppa/_root_pdfs/, leaving 0 unorganized root files. Directly feeds iron ore throughput charts on index.html. Stored in corpus.duckdb.</t>
         </is>
@@ -3367,27 +3463,30 @@
       <c r="O32" s="2" t="n">
         <v>1310</v>
       </c>
-      <c r="P32" s="3" t="inlineStr">
+      <c r="P32" s="3" t="n">
+        <v>1310</v>
+      </c>
+      <c r="Q32" s="3" t="inlineStr">
         <is>
           <t>No (Complete tabular statutory financials, fleet lists, debt notes)</t>
         </is>
       </c>
-      <c r="Q32" s="3" t="inlineStr">
+      <c r="R32" s="3" t="inlineStr">
         <is>
           <t>sec2md HTML DOM parser + standardized YAML frontmatter normalizer</t>
         </is>
       </c>
-      <c r="R32" s="3" t="inlineStr">
+      <c r="S32" s="3" t="inlineStr">
         <is>
           <t>Direct structured Markdown with standardized YAML frontmatter across 26 corporate subdirectories</t>
         </is>
       </c>
-      <c r="S32" s="3" t="inlineStr">
+      <c r="T32" s="3" t="inlineStr">
         <is>
           <t>fetch_sec_filings.py &amp; audit_sec_corpus.py</t>
         </is>
       </c>
-      <c r="T32" s="3" t="inlineStr">
+      <c r="U32" s="3" t="inlineStr">
         <is>
           <t>100% clean Markdown across 26 tickers (VALE, RIO, BHP, FSUGY, SBLK, GOGL, GNK, SB, DSX, SHIP, CTRM, GLBS, EDRY, FRO, INSW, STNG, DHT, TNK, TRMD, ECO, NAT, TNP, ASC, SFL, NVGS, LPG). Zero conversion artifacts. Standardized YAML frontmatter.</t>
         </is>

</xml_diff>

<commit_message>
refactor(audit): unify all markdown under data/extracted/md and update cadence audit
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U32"/>
+  <dimension ref="A1:U33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>corpus/10-companies</t>
+          <t>data/extracted/md/companies</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -3489,6 +3489,99 @@
       <c r="U32" s="3" t="inlineStr">
         <is>
           <t>100% clean Markdown across 26 tickers (VALE, RIO, BHP, FSUGY, SBLK, GOGL, GNK, SB, DSX, SHIP, CTRM, GLBS, EDRY, FRO, INSW, STNG, DHT, TNK, TRMD, ECO, NAT, TNP, ASC, SFL, NVGS, LPG). Zero conversion artifacts. Standardized YAML frontmatter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>maritime_books</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Maritime Reference Literature &amp; Academic Textbooks (12 Books)</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>corpus/books</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>data/extracted/md/books</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Static Reference Corpus</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>CURRENT (1d ago)</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="P33" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>Yes (LaTeX math formulas, figures, port facilities)</t>
+        </is>
+      </c>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>Native GFM normalizer + LaTeX math blocks ($$...$$)</t>
+        </is>
+      </c>
+      <c r="S33" s="3" t="inlineStr">
+        <is>
+          <t>Clean Markdown in data/extracted/md/books/*.md and knowledge/docs/books/*.md</t>
+        </is>
+      </c>
+      <c r="T33" s="3" t="inlineStr">
+        <is>
+          <t>normalize_maritime_books.py</t>
+        </is>
+      </c>
+      <c r="U33" s="3" t="inlineStr">
+        <is>
+          <t>12 foundational academic textbooks and handbooks fully normalized and audited with 100% byte parity in corpus/books/, data/extracted/md/books/, and knowledge/docs/books/.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(pipeline): year-segregate Signal Ocean MDs, fix 184 ld+json dates, wire master pipeline, and ingest 2026-10-05 reports
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1949,19 +1949,19 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (7d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
@@ -1973,10 +1973,10 @@
         <v>0</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="S16" s="3" t="inlineStr">
         <is>
-          <t>star_asia_snp_sales_series.csv (3,575 rows), star_asia_deals_series.csv (3,349 rows), star_asia_valuation_matrix_series.csv (3,232 rows), star_asia_demolition_series.csv (3,120 rows), star_asia_metals_energy_series.csv (1,327 rows)</t>
+          <t>star_asia_snp_sales_series.csv (3,575 rows), star_asia_deals_series.csv (3,354 rows), star_asia_valuation_matrix_series.csv (3,232 rows), star_asia_demolition_series.csv (3,136 rows), star_asia_metals_energy_series.csv (1,327 rows)</t>
         </is>
       </c>
       <c r="T16" s="3" t="inlineStr">
@@ -2150,7 +2150,7 @@
         <v>2141</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="M18" s="2" t="n">
         <v>1210</v>
@@ -2159,10 +2159,10 @@
         <v>0</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>1639</v>
+        <v>1638</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>4159</v>
+        <v>4158</v>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
@@ -2243,7 +2243,7 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="M19" s="2" t="n">
         <v>760</v>
@@ -2252,10 +2252,10 @@
         <v>0</v>
       </c>
       <c r="O19" s="2" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
@@ -2321,19 +2321,19 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>4523</v>
+        <v>4524</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>0</v>
@@ -2345,10 +2345,10 @@
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1190</v>
+        <v>1193</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>4523</v>
+        <v>4524</v>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>corpus/03-breakwave/insights</t>
+          <t>data/extracted/md/breakwave</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -2693,34 +2693,34 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
         <v>304</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>3239</v>
+        <v>3242</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>15083</v>
+        <v>15092</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>3210</v>
+        <v>3213</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>3210</v>
+        <v>3504</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>21836</v>
+        <v>21851</v>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,745 rows), breakwave_insights_metadata.csv (3,210 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,745 rows), breakwave_insights_metadata.csv (3,213 rows)</t>
         </is>
       </c>
       <c r="T24" s="3" t="inlineStr">
@@ -3153,20 +3153,20 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2021-05-14</t>
+          <t>2020-12-29</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (11d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K29" s="2" t="n">
@@ -3179,13 +3179,13 @@
         <v>1494</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="O29" s="2" t="n">
         <v>446</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>2896</v>
+        <v>2891</v>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
@@ -3199,7 +3199,7 @@
       </c>
       <c r="S29" s="3" t="inlineStr">
         <is>
-          <t>signal_reports_metadata.csv (446 rows), data/views/signal/live_fleet_positions.json (9,082 tracked hulls), data/views/signal/port_queues_active.json (1,932 ports)</t>
+          <t>signal_reports_metadata.csv (446 rows), signal_vessel_counts_series.csv (106 rows), data/views/signal/live_fleet_positions.json (9,082 tracked hulls), data/views/signal/port_queues_active.json (1,932 ports)</t>
         </is>
       </c>
       <c r="T29" s="3" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="U29" s="3" t="inlineStr">
         <is>
-          <t>Live automated telemetry syncs active tanker queues and fleet AIS positions.</t>
+          <t>Live automated telemetry syncs active tanker queues and fleet AIS positions. All 446 articles segregated by year across monitors, newsroom, and newsletters.</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>corpus/08-baltic</t>
+          <t>data/extracted/md/baltic</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -3266,19 +3266,19 @@
         <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>3047</v>
+        <v>3048</v>
       </c>
       <c r="M30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>2227</v>
+        <v>2228</v>
       </c>
       <c r="O30" s="2" t="n">
-        <v>2227</v>
+        <v>2228</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>5274</v>
+        <v>5276</v>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t>baltic_reports_metadata.csv (2,227 rows), baltic_ncfi_series.csv (2,036 rows)</t>
+          <t>baltic_reports_metadata.csv (2,228 rows), baltic_ncfi_series.csv (2,036 rows)</t>
         </is>
       </c>
       <c r="T30" s="3" t="inlineStr">

</xml_diff>

<commit_message>
fix(pipeline): resolve all 4 screenshot formatting/table/chart issues and harden Cloudflare/holiday/split-page extraction
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -550,7 +550,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Status (2026-10-05)</t>
+          <t>Status (2026-10-06)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -651,11 +651,11 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (2d ago)</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
@@ -744,11 +744,11 @@
         </is>
       </c>
       <c r="I3" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (2d ago)</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K3" s="2" t="n">
@@ -837,11 +837,11 @@
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
@@ -930,11 +930,11 @@
         </is>
       </c>
       <c r="I5" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (5d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K5" s="2" t="n">
@@ -1023,11 +1023,11 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (7d ago)</t>
+          <t>CURRENT (8d ago)</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
@@ -1209,11 +1209,11 @@
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K8" s="2" t="n">
@@ -1302,11 +1302,11 @@
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K9" s="2" t="n">
@@ -1395,11 +1395,11 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K10" s="2" t="n">
@@ -1488,11 +1488,11 @@
         </is>
       </c>
       <c r="I11" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (10d ago)</t>
+          <t>CURRENT (11d ago)</t>
         </is>
       </c>
       <c r="K11" s="2" t="n">
@@ -1581,11 +1581,11 @@
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (5d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K12" s="2" t="n">
@@ -1674,11 +1674,11 @@
         </is>
       </c>
       <c r="I13" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (7d ago)</t>
+          <t>CURRENT (8d ago)</t>
         </is>
       </c>
       <c r="K13" s="2" t="n">
@@ -1860,11 +1860,11 @@
         </is>
       </c>
       <c r="I15" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (7d ago)</t>
+          <t>CURRENT (8d ago)</t>
         </is>
       </c>
       <c r="K15" s="2" t="n">
@@ -1953,11 +1953,11 @@
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (0d ago)</t>
+          <t>CURRENT (1d ago)</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
@@ -2046,11 +2046,11 @@
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (6d ago)</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">
@@ -2139,11 +2139,11 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (2d ago)</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
@@ -2232,11 +2232,11 @@
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (5d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K19" s="2" t="n">
@@ -2325,11 +2325,11 @@
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (0d ago)</t>
+          <t>CURRENT (1d ago)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="S20" s="3" t="inlineStr">
         <is>
-          <t>hellenic_iron_ore_pdf_brands_series.csv (31,470 rows)</t>
+          <t>hellenic_iron_ore_pdf_brands_series.csv (31,516 rows)</t>
         </is>
       </c>
       <c r="T20" s="3" t="inlineStr">
@@ -2418,11 +2418,11 @@
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (6d ago)</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K21" s="2" t="n">
@@ -2511,11 +2511,11 @@
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (5d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K22" s="2" t="n">
@@ -2604,11 +2604,11 @@
         </is>
       </c>
       <c r="I23" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (6d ago)</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K23" s="2" t="n">
@@ -2697,11 +2697,11 @@
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (0d ago)</t>
+          <t>CURRENT (1d ago)</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
@@ -2790,11 +2790,11 @@
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (7d ago)</t>
+          <t>CURRENT (8d ago)</t>
         </is>
       </c>
       <c r="K25" s="2" t="n">
@@ -2883,11 +2883,11 @@
         </is>
       </c>
       <c r="I26" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>NORMAL INTERVAL (34d ago)</t>
+          <t>NORMAL INTERVAL (35d ago)</t>
         </is>
       </c>
       <c r="K26" s="2" t="n">
@@ -2976,11 +2976,11 @@
         </is>
       </c>
       <c r="I27" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (11d ago)</t>
+          <t>CURRENT (12d ago)</t>
         </is>
       </c>
       <c r="K27" s="2" t="n">
@@ -3069,11 +3069,11 @@
         </is>
       </c>
       <c r="I28" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (4d ago)</t>
+          <t>CURRENT (5d ago)</t>
         </is>
       </c>
       <c r="K28" s="2" t="n">
@@ -3162,11 +3162,11 @@
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (6d ago)</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K29" s="2" t="n">
@@ -3255,11 +3255,11 @@
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K30" s="2" t="n">
@@ -3348,11 +3348,11 @@
         </is>
       </c>
       <c r="I31" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>NORMAL INTERVAL (34d ago)</t>
+          <t>NORMAL INTERVAL (35d ago)</t>
         </is>
       </c>
       <c r="K31" s="2" t="n">
@@ -3441,11 +3441,11 @@
         </is>
       </c>
       <c r="I32" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K32" s="2" t="n">
@@ -3534,11 +3534,11 @@
         </is>
       </c>
       <c r="I33" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d ago)</t>
+          <t>CURRENT (2d ago)</t>
         </is>
       </c>
       <c r="K33" s="2" t="n">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>31,470 rows</t>
+          <t>31,516 rows</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">

</xml_diff>

<commit_message>
fix(pipeline): resolve knowledge validator asset links, book section counts, LlamaParse key pool rotation, and Signal extraction
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="K16" s="2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
@@ -1976,7 +1976,7 @@
         <v>200</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
@@ -3179,13 +3179,13 @@
         <v>1494</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="O29" s="2" t="n">
         <v>446</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>2891</v>
+        <v>2895</v>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-06
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -647,19 +647,19 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>0</v>
@@ -671,10 +671,10 @@
         <v>0</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
       </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>advanced_shipping_sales_series.csv (6,097 rows), advanced_shipping_demolition_series.csv (2,016 rows), advanced_shipping_secondhand_matrix_series.csv (8,078 rows), advanced_shipping_newbuilding_series.csv (1,895 rows), advanced_shipping_demo_sales_series.csv (601 rows)</t>
+          <t>advanced_shipping_sales_series.csv (6,105 rows), advanced_shipping_demolition_series.csv (2,016 rows), advanced_shipping_secondhand_matrix_series.csv (8,110 rows), advanced_shipping_newbuilding_series.csv (1,909 rows), advanced_shipping_demo_sales_series.csv (604 rows)</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr">
@@ -740,19 +740,19 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I3" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K3" s="2" t="n">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>0</v>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
@@ -781,7 +781,7 @@
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>affinity_tce_series.csv (4,039 rows), affinity_bda_series.csv (744 rows), affinity_indices_series.csv (496 rows)</t>
+          <t>affinity_tce_series.csv (4,039 rows), affinity_bda_series.csv (744 rows), affinity_indices_series.csv (490 rows)</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
@@ -833,19 +833,19 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (4d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>0</v>
@@ -857,10 +857,10 @@
         <v>0</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="K5" s="2" t="n">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>0</v>
@@ -950,10 +950,10 @@
         <v>0</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -967,7 +967,7 @@
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>bancosta_freight_rates_series.csv (20,587 rows), bancosta_ffa_series.csv (7,726 rows), bancosta_sales_series.csv (3,220 rows), bancosta_commodities_series.csv (8,555 rows), bancosta_newbuilding_series.csv (2,377 rows), bancosta_secondhand_matrix_series.csv (1,898 rows), bancosta_demolition_series.csv (974 rows)</t>
+          <t>bancosta_freight_rates_series.csv (20,321 rows), bancosta_ffa_series.csv (7,618 rows), bancosta_sales_series.csv (4,591 rows), bancosta_commodities_series.csv (8,447 rows), bancosta_newbuilding_series.csv (1,952 rows), bancosta_secondhand_matrix_series.csv (1,911 rows), bancosta_demolition_series.csv (1,288 rows)</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>carriers_sales_series.csv (3,130 rows), carriers_dry_tc_period_series.csv (3,216 rows), carriers_indices_series.csv (1,876 rows), carriers_tanker_tce_series.csv (804 rows), carriers_bspa_series.csv (749 rows), carriers_newbuilding_series.csv (312 rows), carriers_demolition_series.csv (178 rows)</t>
+          <t>carriers_sales_series.csv (3,004 rows), carriers_dry_tc_period_series.csv (3,072 rows), carriers_indices_series.csv (1,792 rows), carriers_tanker_tce_series.csv (768 rows), carriers_bspa_series.csv (713 rows), carriers_newbuilding_series.csv (301 rows), carriers_demolition_series.csv (171 rows)</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
@@ -1112,19 +1112,19 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (0d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K7" s="2" t="n">
-        <v>11</v>
+        <v>181</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>0</v>
@@ -1136,10 +1136,10 @@
         <v>0</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>11</v>
+        <v>181</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>clarksons_sales_series.csv (1,343 rows)</t>
+          <t>clarksons_sales_series.csv (1,311 sales rows, 120 demo rows)</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="K8" s="2" t="n">
-        <v>263</v>
+        <v>0</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>0</v>
@@ -1229,10 +1229,10 @@
         <v>4742</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>12000</v>
+        <v>4742</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>5005</v>
+        <v>4742</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>fearnleys_rates_series.csv (17,076 rows)</t>
+          <t>fearnleys_rates_series.csv (14,669 rows)</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
@@ -1322,7 +1322,7 @@
         <v>4742</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>11739</v>
+        <v>4742</v>
       </c>
       <c r="P9" s="3" t="n">
         <v>4742</v>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="K10" s="2" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>2826</v>
+        <v>0</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>184</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>3191</v>
+        <v>184</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1496,7 +1496,7 @@
         </is>
       </c>
       <c r="K11" s="2" t="n">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="L11" s="2" t="n">
         <v>167</v>
@@ -1508,10 +1508,10 @@
         <v>0</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>264</v>
+        <v>0</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>276</v>
+        <v>167</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
@@ -1577,19 +1577,19 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (6d ago)</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K12" s="2" t="n">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="L12" s="2" t="n">
         <v>0</v>
@@ -1601,10 +1601,10 @@
         <v>0</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="S12" s="3" t="inlineStr">
         <is>
-          <t>intermodal_baltic_tc_series.csv (20,348 rows), intermodal_tc_rates_series.csv (5,233 rows), intermodal_newbuilding_series.csv (5,084 rows), intermodal_tanker_spot_series.csv (3,885 rows), intermodal_sales_series.csv (3,479 rows), intermodal_demolition_series.csv (2,620 rows)</t>
+          <t>intermodal_baltic_tc_series.csv (20,348 rows), intermodal_tc_rates_series.csv (5,100 rows), intermodal_newbuilding_series.csv (5,058 rows), intermodal_tanker_spot_series.csv (3,879 rows), intermodal_sales_series.csv (3,358 rows), intermodal_demolition_series.csv (2,629 rows)</t>
         </is>
       </c>
       <c r="T12" s="3" t="inlineStr">
@@ -1694,7 +1694,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>115</v>
+        <v>230</v>
       </c>
       <c r="P13" s="3" t="n">
         <v>115</v>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="S13" s="3" t="inlineStr">
         <is>
-          <t>ism_handy_freight_series.csv (17,968 rows), ism_coaster_freight_series.csv (12,462 rows)</t>
+          <t>ism_handy_freight_series.csv (17,629 rows), ism_coaster_freight_series.csv (12,319 rows)</t>
         </is>
       </c>
       <c r="T13" s="3" t="inlineStr">
@@ -1763,19 +1763,19 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (0d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K14" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L14" s="2" t="n">
         <v>0</v>
@@ -1790,7 +1790,7 @@
         <v>48</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="S14" s="3" t="inlineStr">
         <is>
-          <t>lion_deals_series.csv (1,269 rows), lion_sales_series.csv (1,164 rows), lion_demometer_series.csv (564 rows), lion_demolition_series.csv (516 rows), lion_demo_sales_series.csv (105 rows)</t>
+          <t>lion_deals_series.csv (1,212 rows), lion_sales_series.csv (1,192 rows), lion_demometer_series.csv (576 rows), lion_demolition_series.csv (516 rows), lion_demo_sales_series.csv (105 rows)</t>
         </is>
       </c>
       <c r="T14" s="3" t="inlineStr">
@@ -1880,7 +1880,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="P15" s="3" t="n">
         <v>530</v>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="S15" s="3" t="inlineStr">
         <is>
-          <t>ssy_capesize_index_series.csv (8,729 rows), ssy_capesize_series.csv (8,881 rows), ssy_route_rates_series.csv (5,160 rows), ssy_capesize_index_time_series.csv (516 rows)</t>
+          <t>ssy_capesize_index_series.csv (8,881 rows), ssy_capesize_series.csv (8,881 rows), ssy_route_rates_series.csv (5,190 rows), ssy_capesize_index_time_series.csv (519 rows)</t>
         </is>
       </c>
       <c r="T15" s="3" t="inlineStr">
@@ -1949,19 +1949,19 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d ago)</t>
+          <t>CURRENT (11d ago)</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
@@ -1976,7 +1976,7 @@
         <v>200</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="S16" s="3" t="inlineStr">
         <is>
-          <t>star_asia_snp_sales_series.csv (3,575 rows), star_asia_deals_series.csv (3,354 rows), star_asia_valuation_matrix_series.csv (3,232 rows), star_asia_demolition_series.csv (3,136 rows), star_asia_metals_energy_series.csv (1,327 rows)</t>
+          <t>star_asia_snp_sales_series.csv (3,717 rows), star_asia_deals_series.csv (3,327 rows), star_asia_valuation_matrix_series.csv (3,245 rows), star_asia_demolition_series.csv (3,072 rows), star_asia_metals_energy_series.csv (1,327 rows)</t>
         </is>
       </c>
       <c r="T16" s="3" t="inlineStr">
@@ -2042,15 +2042,15 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (7d ago)</t>
+          <t>CURRENT (8d ago)</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="S17" s="3" t="inlineStr">
         <is>
-          <t>xclusiv_secondhand_series.csv (8,529 rows), xclusiv_sales_series.csv (5,542 rows), xclusiv_demolition_series.csv (2,082 rows), xclusiv_newbuilding_prices_series.csv (1,379 rows), xclusiv_newbuilding_orders_series.csv (1,313 rows)</t>
+          <t>xclusiv_secondhand_series.csv (8,593 rows), xclusiv_sales_series.csv (5,713 rows), xclusiv_demolition_series.csv (2,098 rows), xclusiv_newbuilding_prices_series.csv (1,397 rows), xclusiv_newbuilding_orders_series.csv (1,329 rows)</t>
         </is>
       </c>
       <c r="T17" s="3" t="inlineStr">
@@ -2147,22 +2147,22 @@
         </is>
       </c>
       <c r="K18" s="2" t="n">
-        <v>2141</v>
+        <v>1056</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>1210</v>
+        <v>1211</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>1638</v>
+        <v>739</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>4158</v>
+        <v>3077</v>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
@@ -2243,19 +2243,19 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O19" s="2" t="n">
-        <v>265</v>
+        <v>0</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>1038</v>
+        <v>1040</v>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="S19" s="3" t="inlineStr">
         <is>
-          <t>hellenic_alibra_dry_tc_series.csv (6,467 rows)</t>
+          <t>hellenic_alibra_dry_tc_series.csv (6,443 rows)</t>
         </is>
       </c>
       <c r="T19" s="3" t="inlineStr">
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>4524</v>
+        <v>2252</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>0</v>
@@ -2345,10 +2345,10 @@
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1193</v>
+        <v>12</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>4524</v>
+        <v>2252</v>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="S20" s="3" t="inlineStr">
         <is>
-          <t>hellenic_iron_ore_pdf_brands_series.csv (31,516 rows)</t>
+          <t>hellenic_iron_ore_pdf_brands_series.csv (216 rows)</t>
         </is>
       </c>
       <c r="T20" s="3" t="inlineStr">
@@ -2426,7 +2426,7 @@
         </is>
       </c>
       <c r="K21" s="2" t="n">
-        <v>1362</v>
+        <v>677</v>
       </c>
       <c r="L21" s="2" t="n">
         <v>379</v>
@@ -2438,10 +2438,10 @@
         <v>0</v>
       </c>
       <c r="O21" s="2" t="n">
-        <v>165</v>
+        <v>0</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>1921</v>
+        <v>1236</v>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="S21" s="3" t="inlineStr">
         <is>
-          <t>clarksons_snp_sales_series.csv (1,329 rows), clarksons_demolition_sales_series.csv (70 rows), clarksons_macro_series.csv (165 rows), clarksons_desk_talk_series.csv (352 rows)</t>
+          <t>clarksons_snp_sales_series.csv, clarksons_demolition_sales_series.csv, clarksons_macro_series.csv, clarksons_desk_talk_series.csv</t>
         </is>
       </c>
       <c r="T21" s="3" t="inlineStr">
@@ -2531,7 +2531,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="2" t="n">
-        <v>265</v>
+        <v>0</v>
       </c>
       <c r="P22" s="3" t="n">
         <v>1036</v>
@@ -2548,7 +2548,7 @@
       </c>
       <c r="S22" s="3" t="inlineStr">
         <is>
-          <t>hellenic_alibra_tanker_tc_series.csv (7,205 rows)</t>
+          <t>hellenic_alibra_tanker_tc_series.csv (7,177 rows)</t>
         </is>
       </c>
       <c r="T22" s="3" t="inlineStr">
@@ -2641,7 +2641,7 @@
       </c>
       <c r="S23" s="3" t="inlineStr">
         <is>
-          <t>hellenic_vv_matrix_series.csv (12,350 rows), hellenic_vv_sales_series.csv (2,062 rows)</t>
+          <t>hellenic_vv_matrix_series.csv (12,340 rows), hellenic_vv_sales_series.csv (2,062 rows)</t>
         </is>
       </c>
       <c r="T23" s="3" t="inlineStr">
@@ -2711,16 +2711,16 @@
         <v>3242</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>15092</v>
+        <v>15083</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>3213</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>3504</v>
+        <v>3213</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>21851</v>
+        <v>21842</v>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,745 rows), breakwave_insights_metadata.csv (3,213 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,746 rows), breakwave_insights_metadata.csv (3,210 rows)</t>
         </is>
       </c>
       <c r="T24" s="3" t="inlineStr">
@@ -2786,15 +2786,15 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>CURRENT (8d ago)</t>
+        <v>18</v>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>NORMAL INTERVAL (18d ago)</t>
         </is>
       </c>
       <c r="K25" s="2" t="n">
@@ -2813,7 +2813,7 @@
         <v>1087</v>
       </c>
       <c r="P25" s="3" t="n">
-        <v>1087</v>
+        <v>3270</v>
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
@@ -2827,7 +2827,7 @@
       </c>
       <c r="S25" s="3" t="inlineStr">
         <is>
-          <t>poten_opinions_metadata.csv (1,087 rows), poten_top_charterers_series.csv (756 rows), poten_fixtures_series.csv (100 rows)</t>
+          <t>poten_opinions_metadata.csv (1,087 rows), poten_top_charterers_series.csv (755 rows), poten_fixtures_series.csv (100 rows)</t>
         </is>
       </c>
       <c r="T25" s="3" t="inlineStr">
@@ -2891,7 +2891,7 @@
         </is>
       </c>
       <c r="K26" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -2903,10 +2903,10 @@
         <v>99</v>
       </c>
       <c r="O26" s="2" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="P26" s="3" t="n">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="S26" s="3" t="inlineStr">
         <is>
-          <t>seabrokers_osv_monthly_history_series.csv (6,280 rows), seabrokers_rigs_market_series.csv (5,433 rows), seabrokers_osv_utilisation_series.csv (2,304 rows), seabrokers_osv_spot_rates_series.csv (1,855 rows)</t>
+          <t>seabrokers_osv_monthly_history_series.csv (6,280 rows), seabrokers_rigs_market_series.csv (4,467 rows), seabrokers_osv_utilisation_series.csv (2,304 rows), seabrokers_osv_spot_rates_series.csv (1,855 rows)</t>
         </is>
       </c>
       <c r="T26" s="3" t="inlineStr">
@@ -2999,7 +2999,7 @@
         <v>288</v>
       </c>
       <c r="P27" s="3" t="n">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
@@ -3089,7 +3089,7 @@
         <v>1092</v>
       </c>
       <c r="O28" s="2" t="n">
-        <v>551</v>
+        <v>1092</v>
       </c>
       <c r="P28" s="3" t="n">
         <v>1097</v>
@@ -3176,16 +3176,16 @@
         <v>515</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>1494</v>
+        <v>1193</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>450</v>
       </c>
       <c r="O29" s="2" t="n">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>2895</v>
+        <v>2594</v>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t>baltic_reports_metadata.csv (2,228 rows), baltic_ncfi_series.csv (2,036 rows)</t>
+          <t>baltic_reports_metadata.csv (2,227 rows), baltic_ncfi_series.csv (2,180 rows)</t>
         </is>
       </c>
       <c r="T30" s="3" t="inlineStr">
@@ -3344,19 +3344,19 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="I31" s="2" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>NORMAL INTERVAL (35d ago)</t>
+          <t>NORMAL INTERVAL (70d ago)</t>
         </is>
       </c>
       <c r="K31" s="2" t="n">
-        <v>518</v>
+        <v>493</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -3371,7 +3371,7 @@
         <v>0</v>
       </c>
       <c r="P31" s="3" t="n">
-        <v>518</v>
+        <v>493</v>
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
@@ -3928,7 +3928,7 @@
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="47" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="48" customWidth="1" min="9" max="9"/>
   </cols>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows</t>
+          <t>14,768 rows across classes</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows</t>
+          <t>14,768 rows across classes</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows</t>
+          <t>14,768 rows across classes</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows</t>
+          <t>14,768 rows across classes</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows</t>
+          <t>14,768 rows across classes</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows</t>
+          <t>14,768 rows across classes</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows</t>
+          <t>14,768 rows across classes</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows</t>
+          <t>14,768 rows across classes</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -4389,7 +4389,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows</t>
+          <t>14,768 rows across classes</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>14,768 rows</t>
+          <t>14,768 rows across classes</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1,096 rows</t>
+          <t>1,092 rows</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>2,921 rows</t>
+          <t>2,905 rows</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -4765,7 +4765,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>892 rows</t>
+          <t>887 rows (deals), 863 rows (rates)</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>6,467 rows</t>
+          <t>6,443 rows</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>7,205 rows</t>
+          <t>7,177 rows</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>31,516 rows</t>
+          <t>216 rows</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>4,770 rows</t>
+          <t>1,171 rows</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>12,350 rows</t>
+          <t>12,340 rows</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -5235,7 +5235,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>105 rows</t>
+          <t>26 workbook sheets</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>756 rows</t>
+          <t>755 rows (charterers), 1,087 rows (metadata)</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>6,280 rows</t>
+          <t>15,430 rows across 9 series</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>446 rows</t>
+          <t>446 rows + live JSON views</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>5,542 rows</t>
+          <t>17,737 rows across 5 series</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -5470,7 +5470,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>6,097 rows</t>
+          <t>18,744 rows across 5 series</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -5517,7 +5517,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>3,220 rows</t>
+          <t>5,043 rows across 3 series</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>20,348 rows</t>
+          <t>20,348 rows across series</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-07
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="K5" s="2" t="n">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>0</v>
@@ -953,7 +953,7 @@
         <v>251</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c r="K12" s="2" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="L12" s="2" t="n">
         <v>0</v>
@@ -1604,7 +1604,7 @@
         <v>258</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
@@ -1868,7 +1868,7 @@
         </is>
       </c>
       <c r="K15" s="2" t="n">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
         <v>531</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
@@ -2054,7 +2054,7 @@
         </is>
       </c>
       <c r="K17" s="2" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0</v>
@@ -2069,7 +2069,7 @@
         <v>273</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
@@ -2135,22 +2135,22 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (4d ago)</t>
+          <t>CURRENT (1d ago)</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
-        <v>2141</v>
+        <v>2143</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="M18" s="2" t="n">
         <v>1211</v>
@@ -2159,10 +2159,10 @@
         <v>0</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>1641</v>
+        <v>1642</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>4162</v>
+        <v>4165</v>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
@@ -2321,19 +2321,19 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (2d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>4524</v>
+        <v>4528</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>1202</v>
@@ -2345,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1193</v>
+        <v>1197</v>
       </c>
       <c r="P20" s="3" t="n">
         <v>9057</v>
@@ -2414,22 +2414,22 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (8d ago)</t>
+          <t>CURRENT (1d ago)</t>
         </is>
       </c>
       <c r="K21" s="2" t="n">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="M21" s="2" t="n">
         <v>180</v>
@@ -2441,7 +2441,7 @@
         <v>165</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>1921</v>
+        <v>1923</v>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
@@ -2600,22 +2600,22 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="I23" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (8d ago)</t>
+          <t>CURRENT (1d ago)</t>
         </is>
       </c>
       <c r="K23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>733</v>
@@ -2627,7 +2627,7 @@
         <v>261</v>
       </c>
       <c r="P23" s="3" t="n">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="S23" s="3" t="inlineStr">
         <is>
-          <t>hellenic_vv_matrix_series.csv (12,350 rows), hellenic_vv_sales_series.csv (2,062 rows)</t>
+          <t>hellenic_vv_matrix_series.csv (12,350 rows), hellenic_vv_sales_series.csv (2,030 rows)</t>
         </is>
       </c>
       <c r="T23" s="3" t="inlineStr">
@@ -5094,7 +5094,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2,062 rows</t>
+          <t>2,030 rows</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-08
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -2321,19 +2321,19 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>4528</v>
+        <v>4530</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>1202</v>
@@ -2345,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="P20" s="3" t="n">
         <v>9057</v>
@@ -2693,34 +2693,34 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (2d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
         <v>305</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>3243</v>
+        <v>3245</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>15095</v>
+        <v>15102</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>3214</v>
+        <v>3216</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>3506</v>
+        <v>3508</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>21857</v>
+        <v>21868</v>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,755 rows), breakwave_insights_metadata.csv (3,214 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,755 rows), breakwave_insights_metadata.csv (3,216 rows)</t>
         </is>
       </c>
       <c r="T24" s="3" t="inlineStr">
@@ -3266,19 +3266,19 @@
         <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>3048</v>
+        <v>3049</v>
       </c>
       <c r="M30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>2228</v>
+        <v>2229</v>
       </c>
       <c r="O30" s="2" t="n">
-        <v>2228</v>
+        <v>2229</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>5276</v>
+        <v>5278</v>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t>baltic_reports_metadata.csv (2,228 rows), baltic_ncfi_series.csv (2,041 rows)</t>
+          <t>baltic_reports_metadata.csv (2,229 rows), baltic_ncfi_series.csv (2,045 rows)</t>
         </is>
       </c>
       <c r="T30" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-09
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2321,19 +2321,19 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>4530</v>
+        <v>4532</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>1202</v>
@@ -2345,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1199</v>
+        <v>1201</v>
       </c>
       <c r="P20" s="3" t="n">
         <v>9057</v>
@@ -3251,34 +3251,34 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (7d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>3049</v>
+        <v>3054</v>
       </c>
       <c r="M30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>2229</v>
+        <v>2234</v>
       </c>
       <c r="O30" s="2" t="n">
-        <v>2229</v>
+        <v>2234</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>5278</v>
+        <v>5288</v>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t>baltic_reports_metadata.csv (2,229 rows), baltic_ncfi_series.csv (2,045 rows)</t>
+          <t>baltic_reports_metadata.csv (2,234 rows), baltic_ncfi_series.csv (2,049 rows)</t>
         </is>
       </c>
       <c r="T30" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-12
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -2693,34 +2693,34 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (4d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
         <v>305</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>3245</v>
+        <v>3247</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>15102</v>
+        <v>15107</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>3216</v>
+        <v>3218</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>3507</v>
+        <v>3510</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>21868</v>
+        <v>21877</v>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,755 rows), breakwave_insights_metadata.csv (3,216 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,755 rows), breakwave_insights_metadata.csv (3,218 rows)</t>
         </is>
       </c>
       <c r="T24" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Lion: fix nested-paren and mid-line vessel parsing; cadence day parse
run_lion_tables.parse_deal_line dropped "(X" after nested brackets and
merged vessels listed mid-line; price_basis now records each / en bloc.
46+7 MDs, sidecars and the 4 Lion series rebuilt; 1,164 DWT and 1,188
prices verified against the PDFs. Register counts 1,312 deals / 1,203
secondhand sales.

generate_cadence_audit.parse_date_from_filename read "2 October 2026"
style names as the 28th (future dates for Lion/Clarksons/Poten); it now
reads the day, bare months still default to the 28th. Cadence md/xlsx
regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -550,7 +550,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Status (2026-10-12)</t>
+          <t>Status (2026-10-13)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -651,11 +651,11 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (2d ago)</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
@@ -744,11 +744,11 @@
         </is>
       </c>
       <c r="I3" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (2d ago)</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K3" s="2" t="n">
@@ -837,11 +837,11 @@
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
@@ -930,11 +930,11 @@
         </is>
       </c>
       <c r="I5" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (5d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K5" s="2" t="n">
@@ -1023,11 +1023,11 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (5d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
@@ -1112,15 +1112,15 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (0d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K7" s="2" t="n">
@@ -1209,11 +1209,11 @@
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K8" s="2" t="n">
@@ -1302,11 +1302,11 @@
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K9" s="2" t="n">
@@ -1395,11 +1395,11 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (5d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K10" s="2" t="n">
@@ -1488,11 +1488,11 @@
         </is>
       </c>
       <c r="I11" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K11" s="2" t="n">
@@ -1581,11 +1581,11 @@
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (5d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K12" s="2" t="n">
@@ -1674,11 +1674,11 @@
         </is>
       </c>
       <c r="I13" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>CURRENT (14d ago)</t>
+        <v>15</v>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>NORMAL INTERVAL (15d ago)</t>
         </is>
       </c>
       <c r="K13" s="2" t="n">
@@ -1763,15 +1763,15 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (0d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K14" s="2" t="n">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="S14" s="3" t="inlineStr">
         <is>
-          <t>lion_deals_series.csv (1,303 rows), lion_sales_series.csv (1,194 rows), lion_demometer_series.csv (576 rows), lion_demolition_series.csv (516 rows), lion_demo_sales_series.csv (109 rows)</t>
+          <t>lion_deals_series.csv (1,312 rows), lion_sales_series.csv (1,203 rows), lion_demometer_series.csv (576 rows), lion_demolition_series.csv (516 rows), lion_demo_sales_series.csv (109 rows)</t>
         </is>
       </c>
       <c r="T14" s="3" t="inlineStr">
@@ -1860,11 +1860,11 @@
         </is>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (0d ago)</t>
+          <t>CURRENT (1d ago)</t>
         </is>
       </c>
       <c r="K15" s="2" t="n">
@@ -1953,11 +1953,11 @@
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (0d ago)</t>
+          <t>CURRENT (1d ago)</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
@@ -2046,11 +2046,11 @@
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (6d ago)</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">
@@ -2139,11 +2139,11 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (2d ago)</t>
+          <t>CURRENT (3d ago)</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
@@ -2232,11 +2232,11 @@
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (5d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K19" s="2" t="n">
@@ -2325,11 +2325,11 @@
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
@@ -2418,11 +2418,11 @@
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (6d ago)</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K21" s="2" t="n">
@@ -2511,11 +2511,11 @@
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (5d ago)</t>
+          <t>CURRENT (6d ago)</t>
         </is>
       </c>
       <c r="K22" s="2" t="n">
@@ -2604,11 +2604,11 @@
         </is>
       </c>
       <c r="I23" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (6d ago)</t>
+          <t>CURRENT (7d ago)</t>
         </is>
       </c>
       <c r="K23" s="2" t="n">
@@ -2697,11 +2697,11 @@
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (4d ago)</t>
+          <t>CURRENT (5d ago)</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
@@ -2786,15 +2786,15 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (0d ago)</t>
+          <t>CURRENT (11d ago)</t>
         </is>
       </c>
       <c r="K25" s="2" t="n">
@@ -2883,11 +2883,11 @@
         </is>
       </c>
       <c r="I26" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>NORMAL INTERVAL (41d ago)</t>
+          <t>NORMAL INTERVAL (42d ago)</t>
         </is>
       </c>
       <c r="K26" s="2" t="n">
@@ -2976,11 +2976,11 @@
         </is>
       </c>
       <c r="I27" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>NORMAL INTERVAL (18d ago)</t>
+          <t>NORMAL INTERVAL (19d ago)</t>
         </is>
       </c>
       <c r="K27" s="2" t="n">
@@ -3069,11 +3069,11 @@
         </is>
       </c>
       <c r="I28" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (4d ago)</t>
+          <t>CURRENT (5d ago)</t>
         </is>
       </c>
       <c r="K28" s="2" t="n">
@@ -3162,11 +3162,11 @@
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K29" s="2" t="n">
@@ -3255,11 +3255,11 @@
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K30" s="2" t="n">
@@ -3348,11 +3348,11 @@
         </is>
       </c>
       <c r="I31" s="2" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>NORMAL INTERVAL (76d ago)</t>
+          <t>NORMAL INTERVAL (77d ago)</t>
         </is>
       </c>
       <c r="K31" s="2" t="n">
@@ -3441,11 +3441,11 @@
         </is>
       </c>
       <c r="I32" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d ago)</t>
+          <t>CURRENT (4d ago)</t>
         </is>
       </c>
       <c r="K32" s="2" t="n">
@@ -3534,11 +3534,11 @@
         </is>
       </c>
       <c r="I33" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (8d ago)</t>
+          <t>CURRENT (9d ago)</t>
         </is>
       </c>
       <c r="K33" s="2" t="n">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-13
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -688,7 +688,7 @@
       </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>advanced_shipping_sales_series.csv (6,097 rows), advanced_shipping_demolition_series.csv (2,000 rows), advanced_shipping_secondhand_matrix_series.csv (8,093 rows), advanced_shipping_newbuilding_series.csv (1,898 rows), advanced_shipping_demo_sales_series.csv (599 rows)</t>
+          <t>advanced_shipping_sales_series.csv (6,106 rows), advanced_shipping_demolition_series.csv (2,000 rows), advanced_shipping_secondhand_matrix_series.csv (8,093 rows), advanced_shipping_newbuilding_series.csv (1,898 rows), advanced_shipping_demo_sales_series.csv (599 rows)</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr">
@@ -1031,7 +1031,7 @@
         </is>
       </c>
       <c r="K6" s="2" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L6" s="2" t="n">
         <v>0</v>
@@ -1046,7 +1046,7 @@
         <v>137</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -1682,7 +1682,7 @@
         </is>
       </c>
       <c r="K13" s="2" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L13" s="2" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
         <v>230</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
@@ -1868,7 +1868,7 @@
         </is>
       </c>
       <c r="K15" s="2" t="n">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
         <v>531</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="K16" s="2" t="n">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
@@ -1976,7 +1976,7 @@
         <v>200</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
@@ -2054,7 +2054,7 @@
         </is>
       </c>
       <c r="K17" s="2" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0</v>
@@ -2069,7 +2069,7 @@
         <v>271</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
@@ -2321,19 +2321,19 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (4d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>4532</v>
+        <v>4536</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>1202</v>
@@ -2345,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1189</v>
+        <v>1193</v>
       </c>
       <c r="P20" s="3" t="n">
         <v>9057</v>
@@ -2693,34 +2693,34 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>3247</v>
+        <v>3249</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>15107</v>
+        <v>15111</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>3218</v>
+        <v>3220</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>3509</v>
+        <v>3512</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>21877</v>
+        <v>21886</v>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,747 rows), breakwave_insights_metadata.csv (3,218 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,759 rows), breakwave_insights_metadata.csv (3,220 rows)</t>
         </is>
       </c>
       <c r="T24" s="3" t="inlineStr">
@@ -5470,7 +5470,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>6,097 rows</t>
+          <t>6,106 rows</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-14
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="K5" s="2" t="n">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>0</v>
@@ -953,7 +953,7 @@
         <v>250</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -1391,15 +1391,15 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (7d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K10" s="2" t="n">
@@ -1412,13 +1412,13 @@
         <v>2847</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="O10" s="2" t="n">
         <v>184</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>3215</v>
+        <v>3216</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c r="K12" s="2" t="n">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="L12" s="2" t="n">
         <v>0</v>
@@ -1604,7 +1604,7 @@
         <v>257</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
@@ -2321,19 +2321,19 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>4536</v>
+        <v>4538</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>1202</v>
@@ -2345,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1193</v>
+        <v>1195</v>
       </c>
       <c r="P20" s="3" t="n">
         <v>9057</v>
@@ -2693,34 +2693,34 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
         <v>306</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>3249</v>
+        <v>3251</v>
       </c>
       <c r="M24" s="2" t="n">
         <v>15111</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>3220</v>
+        <v>3222</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>3512</v>
+        <v>3514</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>21886</v>
+        <v>21890</v>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,759 rows), breakwave_insights_metadata.csv (3,220 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,759 rows), breakwave_insights_metadata.csv (3,222 rows)</t>
         </is>
       </c>
       <c r="T24" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-15
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="K8" s="2" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>0</v>
@@ -1232,7 +1232,7 @@
         <v>5036</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>5030</v>
+        <v>5031</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -2228,34 +2228,34 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (8d ago)</t>
+          <t>CURRENT (1d ago)</t>
         </is>
       </c>
       <c r="K19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O19" s="2" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>1042</v>
+        <v>1044</v>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
@@ -2321,19 +2321,19 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>4538</v>
+        <v>4540</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>1202</v>
@@ -2345,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1195</v>
+        <v>1197</v>
       </c>
       <c r="P20" s="3" t="n">
         <v>9057</v>
@@ -2507,34 +2507,34 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (8d ago)</t>
+          <t>CURRENT (1d ago)</t>
         </is>
       </c>
       <c r="K22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O22" s="2" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>1039</v>
+        <v>1041</v>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
@@ -2600,22 +2600,22 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="I23" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (9d ago)</t>
+          <t>CURRENT (1d ago)</t>
         </is>
       </c>
       <c r="K23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>733</v>
@@ -2627,7 +2627,7 @@
         <v>261</v>
       </c>
       <c r="P23" s="3" t="n">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="S23" s="3" t="inlineStr">
         <is>
-          <t>hellenic_vv_matrix_series.csv (12,373 rows), hellenic_vv_sales_series.csv (2,067 rows)</t>
+          <t>hellenic_vv_matrix_series.csv (12,373 rows), hellenic_vv_sales_series.csv (2,077 rows)</t>
         </is>
       </c>
       <c r="T23" s="3" t="inlineStr">
@@ -2693,34 +2693,34 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
         <v>306</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>3251</v>
+        <v>3252</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>15111</v>
+        <v>15113</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>3222</v>
+        <v>3223</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>3514</v>
+        <v>3515</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>21890</v>
+        <v>21894</v>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,759 rows), breakwave_insights_metadata.csv (3,222 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,759 rows), breakwave_insights_metadata.csv (3,223 rows)</t>
         </is>
       </c>
       <c r="T24" s="3" t="inlineStr">
@@ -5094,7 +5094,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2,067 rows</t>
+          <t>2,077 rows</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-16
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2321,19 +2321,19 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>4540</v>
+        <v>4542</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>1202</v>
@@ -2345,7 +2345,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="P20" s="3" t="n">
         <v>9057</v>
@@ -2693,34 +2693,34 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
         <v>306</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>3252</v>
+        <v>3254</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>15113</v>
+        <v>15120</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>3223</v>
+        <v>3225</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>3515</v>
+        <v>3517</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>21894</v>
+        <v>21905</v>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,759 rows), breakwave_insights_metadata.csv (3,223 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,759 rows), breakwave_insights_metadata.csv (3,225 rows)</t>
         </is>
       </c>
       <c r="T24" s="3" t="inlineStr">
@@ -3251,34 +3251,34 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (7d ago)</t>
+          <t>CURRENT (0d ago)</t>
         </is>
       </c>
       <c r="K30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>3054</v>
+        <v>3059</v>
       </c>
       <c r="M30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>2234</v>
+        <v>2239</v>
       </c>
       <c r="O30" s="2" t="n">
-        <v>2234</v>
+        <v>2239</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>5288</v>
+        <v>5298</v>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t>baltic_reports_metadata.csv (2,234 rows), baltic_ncfi_series.csv (2,049 rows)</t>
+          <t>baltic_reports_metadata.csv (2,239 rows), baltic_ncfi_series.csv (2,053 rows)</t>
         </is>
       </c>
       <c r="T30" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Registry: corpus/books is the GraphRAG input; knowledge/docs/books marked legacy, parity claims removed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1488,21 +1488,21 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (5d)</t>
+          <t>CURRENT (3d)</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M9" s="2" t="n">
@@ -1530,7 +1530,7 @@
         <v>4764</v>
       </c>
       <c r="U9" s="2" t="n">
-        <v>4774</v>
+        <v>4775</v>
       </c>
       <c r="V9" s="2" t="n">
         <v>4764</v>
@@ -3119,7 +3119,7 @@
         <v>0</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="O23" s="2" t="n">
         <v>0</v>
@@ -4287,7 +4287,7 @@
       </c>
       <c r="Y33" s="3" t="inlineStr">
         <is>
-          <t>Clean Markdown in data/extracted/md/books/*.md and knowledge/docs/books/*.md</t>
+          <t>Normalized Markdown in corpus/books/*.md (no series; text corpus)</t>
         </is>
       </c>
       <c r="Z33" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-19
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -726,7 +726,7 @@
         <v>0</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="R2" s="2" t="n">
         <v>0</v>
@@ -741,7 +741,7 @@
         <v>253</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="W2" s="3" t="inlineStr">
         <is>
@@ -841,7 +841,7 @@
         <v>0</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="R3" s="2" t="n">
         <v>0</v>
@@ -856,7 +856,7 @@
         <v>250</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="W3" s="3" t="inlineStr">
         <is>
@@ -1301,7 +1301,7 @@
         <v>0</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R7" s="2" t="n">
         <v>0</v>
@@ -1316,7 +1316,7 @@
         <v>10</v>
       </c>
       <c r="V7" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="W7" s="3" t="inlineStr">
         <is>
@@ -2102,7 +2102,7 @@
         <v>0</v>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="R14" s="2" t="n">
         <v>0</v>
@@ -2117,7 +2117,7 @@
         <v>49</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W14" s="3" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
         <v>0</v>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="R15" s="2" t="n">
         <v>0</v>
@@ -2232,7 +2232,7 @@
         <v>522</v>
       </c>
       <c r="V15" s="2" t="n">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="W15" s="3" t="inlineStr">
         <is>
@@ -2332,7 +2332,7 @@
         <v>0</v>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="R16" s="2" t="n">
         <v>0</v>
@@ -2347,7 +2347,7 @@
         <v>199</v>
       </c>
       <c r="V16" s="2" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="W16" s="3" t="inlineStr">
         <is>
@@ -2528,32 +2528,32 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (9d)</t>
+          <t>CURRENT (2d)</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O18" s="2" t="n">
         <v>0</v>
@@ -2562,22 +2562,22 @@
         <v>0</v>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>2147</v>
+        <v>2151</v>
       </c>
       <c r="R18" s="2" t="n">
-        <v>813</v>
+        <v>815</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>1212</v>
+        <v>1213</v>
       </c>
       <c r="T18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U18" s="2" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="V18" s="2" t="n">
-        <v>4172</v>
+        <v>4179</v>
       </c>
       <c r="W18" s="3" t="inlineStr">
         <is>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="Y18" s="3" t="inlineStr">
         <is>
-          <t>athenian_indicative_demolition_series.csv (3,064 rows), hellenic_gms_port_positions_series.csv (3,014 rows), hellenic_gms_demolition_series.csv (1,104 rows), hellenic_best_oasis_deals_series.csv (905 rows), hellenic_best_oasis_demolition_series.csv (866 rows)</t>
+          <t>athenian_indicative_demolition_series.csv (3,064 rows), hellenic_gms_port_positions_series.csv (3,029 rows), hellenic_gms_demolition_series.csv (1,108 rows), hellenic_best_oasis_deals_series.csv (905 rows), hellenic_best_oasis_demolition_series.csv (866 rows)</t>
         </is>
       </c>
       <c r="Z18" s="3" t="inlineStr">
@@ -2758,32 +2758,32 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>4542</v>
+        <v>4544</v>
       </c>
       <c r="R20" s="2" t="n">
         <v>0</v>
@@ -2804,10 +2804,10 @@
         <v>0</v>
       </c>
       <c r="U20" s="2" t="n">
-        <v>1190</v>
+        <v>1201</v>
       </c>
       <c r="V20" s="2" t="n">
-        <v>4542</v>
+        <v>4544</v>
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
@@ -3218,25 +3218,25 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="M24" s="2" t="n">
@@ -3255,19 +3255,19 @@
         <v>306</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>3254</v>
+        <v>3256</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>15120</v>
+        <v>15122</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>3225</v>
+        <v>3227</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>3517</v>
+        <v>3519</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>21905</v>
+        <v>21911</v>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,759 rows), breakwave_insights_metadata.csv (3,225 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,759 rows), breakwave_insights_metadata.csv (3,227 rows)</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1,104 rows</t>
+          <t>1,108 rows</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -5418,7 +5418,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>3,014 rows</t>
+          <t>3,029 rows</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-20
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2758,32 +2758,32 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>4544</v>
+        <v>4546</v>
       </c>
       <c r="R20" s="2" t="n">
         <v>0</v>
@@ -2804,10 +2804,10 @@
         <v>0</v>
       </c>
       <c r="U20" s="2" t="n">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="V20" s="2" t="n">
-        <v>4544</v>
+        <v>4546</v>
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
@@ -3255,19 +3255,19 @@
         <v>307</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>3256</v>
+        <v>3258</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>15122</v>
+        <v>15128</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>3227</v>
+        <v>3229</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>3520</v>
+        <v>3522</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>21912</v>
+        <v>21922</v>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,769 rows), breakwave_insights_metadata.csv (3,227 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,769 rows), breakwave_insights_metadata.csv (3,229 rows)</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-21
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2758,32 +2758,32 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>3545</v>
+        <v>3547</v>
       </c>
       <c r="R20" s="2" t="n">
         <v>0</v>
@@ -2804,10 +2804,10 @@
         <v>0</v>
       </c>
       <c r="U20" s="2" t="n">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="V20" s="2" t="n">
-        <v>3545</v>
+        <v>3547</v>
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
@@ -3218,25 +3218,25 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="M24" s="2" t="n">
@@ -3255,19 +3255,19 @@
         <v>307</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>3258</v>
+        <v>3260</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>15128</v>
+        <v>15129</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>3229</v>
+        <v>3231</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>3522</v>
+        <v>3524</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>21922</v>
+        <v>21927</v>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,769 rows), breakwave_insights_metadata.csv (3,229 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,769 rows), breakwave_insights_metadata.csv (3,231 rows)</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-22
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -2758,32 +2758,32 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>3547</v>
+        <v>3549</v>
       </c>
       <c r="R20" s="2" t="n">
         <v>0</v>
@@ -2804,10 +2804,10 @@
         <v>0</v>
       </c>
       <c r="U20" s="2" t="n">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="V20" s="2" t="n">
-        <v>3547</v>
+        <v>3549</v>
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
@@ -3218,25 +3218,25 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="M24" s="2" t="n">
@@ -3255,19 +3255,19 @@
         <v>307</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>3260</v>
+        <v>3262</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>15129</v>
+        <v>15132</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>3231</v>
+        <v>3233</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>3524</v>
+        <v>3526</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>21927</v>
+        <v>21934</v>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,769 rows), breakwave_insights_metadata.csv (3,231 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,769 rows), breakwave_insights_metadata.csv (3,233 rows)</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-23
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2758,32 +2758,32 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>3549</v>
+        <v>3551</v>
       </c>
       <c r="R20" s="2" t="n">
         <v>0</v>
@@ -2804,10 +2804,10 @@
         <v>0</v>
       </c>
       <c r="U20" s="2" t="n">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="V20" s="2" t="n">
-        <v>3549</v>
+        <v>3551</v>
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
@@ -3140,7 +3140,7 @@
         <v>0</v>
       </c>
       <c r="R23" s="2" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="S23" s="2" t="n">
         <v>733</v>
@@ -3152,7 +3152,7 @@
         <v>258</v>
       </c>
       <c r="V23" s="2" t="n">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="W23" s="3" t="inlineStr">
         <is>
@@ -3218,25 +3218,25 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M24" s="2" t="n">
@@ -3255,19 +3255,19 @@
         <v>307</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>3262</v>
+        <v>3264</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>15132</v>
+        <v>15135</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>3233</v>
+        <v>3235</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>3526</v>
+        <v>3528</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>21934</v>
+        <v>21941</v>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,769 rows), breakwave_insights_metadata.csv (3,233 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,769 rows), breakwave_insights_metadata.csv (3,235 rows)</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">
@@ -3900,32 +3900,32 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (7d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>24.5</v>
+        <v>24.6</v>
       </c>
       <c r="O30" s="2" t="n">
         <v>0</v>
@@ -3937,19 +3937,19 @@
         <v>0</v>
       </c>
       <c r="R30" s="2" t="n">
-        <v>3059</v>
+        <v>3060</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T30" s="2" t="n">
-        <v>2239</v>
+        <v>2240</v>
       </c>
       <c r="U30" s="2" t="n">
-        <v>2239</v>
+        <v>2240</v>
       </c>
       <c r="V30" s="2" t="n">
-        <v>5298</v>
+        <v>5300</v>
       </c>
       <c r="W30" s="3" t="inlineStr">
         <is>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="Y30" s="3" t="inlineStr">
         <is>
-          <t>baltic_reports_metadata.csv (2,239 rows), baltic_ncfi_series.csv (2,053 rows)</t>
+          <t>baltic_reports_metadata.csv (2,240 rows), baltic_ncfi_series.csv (2,057 rows)</t>
         </is>
       </c>
       <c r="Z30" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-26
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2519,32 +2519,32 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (6d)</t>
+          <t>CURRENT (2d)</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="M18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O18" s="2" t="n">
         <v>0</v>
@@ -2553,22 +2553,22 @@
         <v>0</v>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>1949</v>
+        <v>1953</v>
       </c>
       <c r="R18" s="2" t="n">
-        <v>816</v>
+        <v>818</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>1213</v>
+        <v>1214</v>
       </c>
       <c r="T18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U18" s="2" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="V18" s="2" t="n">
-        <v>3978</v>
+        <v>3985</v>
       </c>
       <c r="W18" s="3" t="inlineStr">
         <is>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="Y18" s="3" t="inlineStr">
         <is>
-          <t>athenian_indicative_demolition_series.csv (3,076 rows), hellenic_gms_port_positions_series.csv (3,029 rows), hellenic_gms_demolition_series.csv (1,108 rows), hellenic_best_oasis_deals_series.csv (905 rows), hellenic_best_oasis_demolition_series.csv (866 rows)</t>
+          <t>athenian_indicative_demolition_series.csv (3,076 rows), hellenic_gms_port_positions_series.csv (3,041 rows), hellenic_gms_demolition_series.csv (1,112 rows), hellenic_best_oasis_deals_series.csv (905 rows), hellenic_best_oasis_demolition_series.csv (866 rows)</t>
         </is>
       </c>
       <c r="Z18" s="3" t="inlineStr">
@@ -2749,32 +2749,32 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>2.2</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>0</v>
@@ -2783,7 +2783,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>3551</v>
+        <v>3553</v>
       </c>
       <c r="R20" s="2" t="n">
         <v>0</v>
@@ -2795,10 +2795,10 @@
         <v>0</v>
       </c>
       <c r="U20" s="2" t="n">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="V20" s="2" t="n">
-        <v>3551</v>
+        <v>3553</v>
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="Y20" s="3" t="inlineStr">
         <is>
-          <t>hellenic_iron_ore_pdf_brands_series.csv (32,482 rows)</t>
+          <t>hellenic_iron_ore_pdf_brands_series.csv (32,502 rows)</t>
         </is>
       </c>
       <c r="Z20" s="3" t="inlineStr">
@@ -3019,7 +3019,7 @@
         <v>282</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="T22" s="2" t="n">
         <v>0</v>
@@ -3028,7 +3028,7 @@
         <v>268</v>
       </c>
       <c r="V22" s="2" t="n">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="W22" s="3" t="inlineStr">
         <is>
@@ -3209,25 +3209,25 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (3d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="M24" s="2" t="n">
@@ -3246,19 +3246,19 @@
         <v>307</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>3264</v>
+        <v>3266</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>15135</v>
+        <v>15137</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>3235</v>
+        <v>3237</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>3528</v>
+        <v>3530</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>21941</v>
+        <v>21947</v>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
@@ -3272,7 +3272,7 @@
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,769 rows), breakwave_insights_metadata.csv (3,235 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,769 rows), breakwave_insights_metadata.csv (3,237 rows)</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">
@@ -5362,7 +5362,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1,108 rows</t>
+          <t>1,112 rows</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -5409,7 +5409,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>3,029 rows</t>
+          <t>3,041 rows</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -5597,7 +5597,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>32,482 rows</t>
+          <t>32,502 rows</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -5644,7 +5644,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>1,193 rows</t>
+          <t>1,194 rows</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-27
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2758,32 +2758,32 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>3553</v>
+        <v>3555</v>
       </c>
       <c r="R20" s="2" t="n">
         <v>0</v>
@@ -2804,10 +2804,10 @@
         <v>0</v>
       </c>
       <c r="U20" s="2" t="n">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="V20" s="2" t="n">
-        <v>3553</v>
+        <v>3555</v>
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="Y20" s="3" t="inlineStr">
         <is>
-          <t>hellenic_iron_ore_pdf_brands_series.csv (32,502 rows)</t>
+          <t>hellenic_iron_ore_pdf_brands_series.csv (32,522 rows)</t>
         </is>
       </c>
       <c r="Z20" s="3" t="inlineStr">
@@ -3255,19 +3255,19 @@
         <v>308</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>3266</v>
+        <v>3267</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>15137</v>
+        <v>15140</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>3237</v>
+        <v>3238</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>3531</v>
+        <v>3532</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>21948</v>
+        <v>21953</v>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,781 rows), breakwave_insights_metadata.csv (3,237 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,781 rows), breakwave_insights_metadata.csv (3,238 rows)</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">
@@ -5606,7 +5606,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>32,502 rows</t>
+          <t>32,522 rows</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -5653,7 +5653,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>1,194 rows</t>
+          <t>1,195 rows</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-28
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1651,13 +1651,13 @@
         <v>2869</v>
       </c>
       <c r="T10" s="2" t="n">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="U10" s="2" t="n">
         <v>186</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>3241</v>
+        <v>3242</v>
       </c>
       <c r="W10" s="3" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
         <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>0</v>
@@ -3218,25 +3218,25 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M24" s="2" t="n">
@@ -3255,19 +3255,19 @@
         <v>308</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>3267</v>
+        <v>3269</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>15140</v>
+        <v>15146</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>3238</v>
+        <v>3240</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>3532</v>
+        <v>3534</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>21953</v>
+        <v>21963</v>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,781 rows), breakwave_insights_metadata.csv (3,238 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,781 rows), breakwave_insights_metadata.csv (3,240 rows)</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-29
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -2643,32 +2643,32 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (8d)</t>
+          <t>CURRENT (1d)</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="O19" s="2" t="n">
         <v>0</v>
@@ -2680,19 +2680,19 @@
         <v>0</v>
       </c>
       <c r="R19" s="2" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="S19" s="2" t="n">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="T19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U19" s="2" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="V19" s="2" t="n">
-        <v>1046</v>
+        <v>1049</v>
       </c>
       <c r="W19" s="3" t="inlineStr">
         <is>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="Y19" s="3" t="inlineStr">
         <is>
-          <t>hellenic_alibra_dry_tc_series.csv (6,587 rows)</t>
+          <t>hellenic_alibra_dry_tc_series.csv (6,611 rows)</t>
         </is>
       </c>
       <c r="Z19" s="3" t="inlineStr">
@@ -2758,32 +2758,32 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (2d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>3555</v>
+        <v>3559</v>
       </c>
       <c r="R20" s="2" t="n">
         <v>0</v>
@@ -2804,10 +2804,10 @@
         <v>0</v>
       </c>
       <c r="U20" s="2" t="n">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="V20" s="2" t="n">
-        <v>3555</v>
+        <v>3559</v>
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="Y20" s="3" t="inlineStr">
         <is>
-          <t>hellenic_iron_ore_pdf_brands_series.csv (32,522 rows)</t>
+          <t>hellenic_iron_ore_pdf_brands_series.csv (32,562 rows)</t>
         </is>
       </c>
       <c r="Z20" s="3" t="inlineStr">
@@ -2988,32 +2988,32 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (8d)</t>
+          <t>CURRENT (1d)</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="M22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="O22" s="2" t="n">
         <v>0</v>
@@ -3025,19 +3025,19 @@
         <v>0</v>
       </c>
       <c r="R22" s="2" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="T22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U22" s="2" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="V22" s="2" t="n">
-        <v>1044</v>
+        <v>1047</v>
       </c>
       <c r="W22" s="3" t="inlineStr">
         <is>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="Y22" s="3" t="inlineStr">
         <is>
-          <t>hellenic_alibra_tanker_tc_series.csv (7,504 rows)</t>
+          <t>hellenic_alibra_tanker_tc_series.csv (7,532 rows)</t>
         </is>
       </c>
       <c r="Z22" s="3" t="inlineStr">
@@ -3218,25 +3218,25 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="M24" s="2" t="n">
@@ -3255,19 +3255,19 @@
         <v>308</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>3269</v>
+        <v>3271</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>15146</v>
+        <v>15153</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>3240</v>
+        <v>3242</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>3534</v>
+        <v>3536</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>21963</v>
+        <v>21974</v>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,781 rows), breakwave_insights_metadata.csv (3,240 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,781 rows), breakwave_insights_metadata.csv (3,242 rows)</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>6,587 rows</t>
+          <t>6,611 rows</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>7,504 rows</t>
+          <t>7,532 rows</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -5606,7 +5606,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>32,522 rows</t>
+          <t>32,562 rows</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -5653,7 +5653,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>1,195 rows</t>
+          <t>1,197 rows</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">

</xml_diff>

<commit_message>
reports: ingest latest market reports and update cadence audit 2026-10-30
</commit_message>
<xml_diff>
--- a/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
+++ b/corpus/CORPUS_PUBLICATION_CADENCE_AND_AUDIT.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corpus Cadence &amp; Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphic &amp; Chart Extraction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sub-Sector &amp; Fleet Breakdown" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1651,13 +1651,13 @@
         <v>2904</v>
       </c>
       <c r="T10" s="2" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U10" s="2" t="n">
         <v>189</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>3282</v>
+        <v>3283</v>
       </c>
       <c r="W10" s="3" t="inlineStr">
         <is>
@@ -2758,32 +2758,32 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>3559</v>
+        <v>3561</v>
       </c>
       <c r="R20" s="2" t="n">
         <v>0</v>
@@ -2804,10 +2804,10 @@
         <v>0</v>
       </c>
       <c r="U20" s="2" t="n">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="V20" s="2" t="n">
-        <v>3559</v>
+        <v>3561</v>
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="Y20" s="3" t="inlineStr">
         <is>
-          <t>hellenic_iron_ore_pdf_brands_series.csv (32,562 rows)</t>
+          <t>hellenic_iron_ore_pdf_brands_series.csv (32,582 rows)</t>
         </is>
       </c>
       <c r="Z20" s="3" t="inlineStr">
@@ -3218,25 +3218,25 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (1d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M24" s="2" t="n">
@@ -3255,19 +3255,19 @@
         <v>308</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>3271</v>
+        <v>3273</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>15153</v>
+        <v>15156</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>3242</v>
+        <v>3244</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>3536</v>
+        <v>3538</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>21974</v>
+        <v>21981</v>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>breakwave_fundamentals_series.csv (2,781 rows), breakwave_insights_metadata.csv (3,242 rows)</t>
+          <t>breakwave_fundamentals_series.csv (2,781 rows), breakwave_insights_metadata.csv (3,244 rows)</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">
@@ -3900,25 +3900,25 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>CURRENT (7d)</t>
+          <t>CURRENT (0d)</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="M30" s="2" t="n">
@@ -3937,19 +3937,19 @@
         <v>0</v>
       </c>
       <c r="R30" s="2" t="n">
-        <v>3064</v>
+        <v>3069</v>
       </c>
       <c r="S30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T30" s="2" t="n">
-        <v>2244</v>
+        <v>2249</v>
       </c>
       <c r="U30" s="2" t="n">
-        <v>2244</v>
+        <v>2249</v>
       </c>
       <c r="V30" s="2" t="n">
-        <v>5308</v>
+        <v>5318</v>
       </c>
       <c r="W30" s="3" t="inlineStr">
         <is>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="Y30" s="3" t="inlineStr">
         <is>
-          <t>baltic_reports_metadata.csv (2,244 rows), baltic_ncfi_series.csv (2,057 rows)</t>
+          <t>baltic_reports_metadata.csv (2,249 rows), baltic_ncfi_series.csv (2,061 rows)</t>
         </is>
       </c>
       <c r="Z30" s="3" t="inlineStr">
@@ -5606,7 +5606,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>32,562 rows</t>
+          <t>32,582 rows</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -5653,7 +5653,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>1,197 rows</t>
+          <t>1,198 rows</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">

</xml_diff>